<commit_message>
Add scripts for generating feature importance rankings and heatmaps
- Introduced `make_missing_feature_correlation_heatmap.py` to create a heatmap including reversible capacity based on updated correlation matrices.
- Added `make_multimodel_rank_supplement.py` to compute and save feature rankings for Linear, Lasso, and Neural Network models, integrating with existing SHAP summaries for RF, GBR, XGB, and Ridge.
- Generated new CSV files for permutation importance rankings and mean absolute SHAP values, enhancing the analysis of model feature importance.
- Outputs are saved in structured directories for easy access and visualization.
</commit_message>
<xml_diff>
--- a/results/reviewer_extension_fixed/missing_feature_analysis/missing_feature_math_analysis/missing_feature_math_analysis.xlsx
+++ b/results/reviewer_extension_fixed/missing_feature_analysis/missing_feature_math_analysis/missing_feature_math_analysis.xlsx
@@ -662,7 +662,7 @@
         <v>524</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.06742782742250555</v>
+        <v>-0.06742782742250554</v>
       </c>
       <c r="G2" t="n">
         <v>0.1231800014169101</v>
@@ -671,7 +671,7 @@
         <v>-0.1371074757307379</v>
       </c>
       <c r="I2" t="n">
-        <v>0.001655725342267778</v>
+        <v>0.001655725342267775</v>
       </c>
       <c r="J2" t="n">
         <v>-0.1045695793933987</v>
@@ -714,7 +714,7 @@
         <v>-0.1524472207635033</v>
       </c>
       <c r="I3" t="n">
-        <v>0.0004620720505100557</v>
+        <v>0.0004620720505100558</v>
       </c>
       <c r="J3" t="n">
         <v>-0.1151604344752149</v>
@@ -757,7 +757,7 @@
         <v>-0.05809852362754963</v>
       </c>
       <c r="I4" t="n">
-        <v>0.268251200131539</v>
+        <v>0.2682512001315391</v>
       </c>
       <c r="J4" t="n">
         <v>-0.0441530581841631</v>
@@ -800,7 +800,7 @@
         <v>-0.0816822071140134</v>
       </c>
       <c r="I5" t="n">
-        <v>0.1192835859700816</v>
+        <v>0.1192835859700817</v>
       </c>
       <c r="J5" t="n">
         <v>-0.06363017915856511</v>
@@ -843,7 +843,7 @@
         <v>-0.6933427652186777</v>
       </c>
       <c r="I6" t="n">
-        <v>1.349719311522128e-44</v>
+        <v>1.349719311522112e-44</v>
       </c>
       <c r="J6" t="n">
         <v>-0.514946747902482</v>
@@ -877,16 +877,16 @@
         <v>302</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.5068825166502335</v>
+        <v>-0.5068825166502333</v>
       </c>
       <c r="G7" t="n">
-        <v>4.059895449149044e-21</v>
+        <v>4.059895449149229e-21</v>
       </c>
       <c r="H7" t="n">
         <v>-0.6543601829456029</v>
       </c>
       <c r="I7" t="n">
-        <v>2.712540233230457e-38</v>
+        <v>2.712540233230541e-38</v>
       </c>
       <c r="J7" t="n">
         <v>-0.4830633699933283</v>
@@ -920,7 +920,7 @@
         <v>286</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1883759717344395</v>
+        <v>0.1883759717344396</v>
       </c>
       <c r="G8" t="n">
         <v>0.001372009608555396</v>
@@ -929,7 +929,7 @@
         <v>0.1025869439101235</v>
       </c>
       <c r="I8" t="n">
-        <v>0.08329551112644691</v>
+        <v>0.0832955111264469</v>
       </c>
       <c r="J8" t="n">
         <v>0.0710620341866106</v>
@@ -972,7 +972,7 @@
         <v>0.1161156691107151</v>
       </c>
       <c r="I9" t="n">
-        <v>0.04979336375797689</v>
+        <v>0.04979336375797688</v>
       </c>
       <c r="J9" t="n">
         <v>0.07607623075020999</v>
@@ -1006,7 +1006,7 @@
         <v>256</v>
       </c>
       <c r="F10" t="n">
-        <v>0.1503119518056599</v>
+        <v>0.15031195180566</v>
       </c>
       <c r="G10" t="n">
         <v>0.01608804321031551</v>
@@ -1015,7 +1015,7 @@
         <v>0.1681245669226088</v>
       </c>
       <c r="I10" t="n">
-        <v>0.007016796862992602</v>
+        <v>0.007016796862992614</v>
       </c>
       <c r="J10" t="n">
         <v>0.1171416007417869</v>
@@ -1049,7 +1049,7 @@
         <v>256</v>
       </c>
       <c r="F11" t="n">
-        <v>0.2266734618594218</v>
+        <v>0.2266734618594217</v>
       </c>
       <c r="G11" t="n">
         <v>0.0002554454456974599</v>
@@ -1058,7 +1058,7 @@
         <v>0.231154352351584</v>
       </c>
       <c r="I11" t="n">
-        <v>0.0001907017655417267</v>
+        <v>0.0001907017655417275</v>
       </c>
       <c r="J11" t="n">
         <v>0.1625391139401165</v>
@@ -1158,10 +1158,10 @@
         <v>524</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.007535451114606645</v>
+        <v>-0.007535451114606691</v>
       </c>
       <c r="G2" t="n">
-        <v>0.1231800014169119</v>
+        <v>0.1231800014169084</v>
       </c>
       <c r="H2" t="n">
         <v>0.7033004313082087</v>
@@ -1201,16 +1201,16 @@
         <v>-6.197844564068472</v>
       </c>
       <c r="G3" t="n">
-        <v>0.01720181667019025</v>
+        <v>0.01720181667018992</v>
       </c>
       <c r="H3" t="n">
-        <v>132.9081403216803</v>
+        <v>132.9081403216805</v>
       </c>
       <c r="I3" t="n">
-        <v>0.01082432276715806</v>
+        <v>0.01082432276715828</v>
       </c>
       <c r="J3" t="n">
-        <v>0.008929350205409303</v>
+        <v>0.008929350205409525</v>
       </c>
     </row>
     <row r="4">
@@ -1238,19 +1238,19 @@
         <v>365</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.007579808508899435</v>
+        <v>-0.007579808508899418</v>
       </c>
       <c r="G4" t="n">
-        <v>0.04944856133872286</v>
+        <v>0.04944856133872343</v>
       </c>
       <c r="H4" t="n">
-        <v>0.7095429265731655</v>
+        <v>0.7095429265731659</v>
       </c>
       <c r="I4" t="n">
-        <v>0.0105919243883551</v>
+        <v>0.01059192438835466</v>
       </c>
       <c r="J4" t="n">
-        <v>0.007866282306780437</v>
+        <v>0.007866282306779993</v>
       </c>
     </row>
     <row r="5">
@@ -1281,16 +1281,16 @@
         <v>-4.097367239884447</v>
       </c>
       <c r="G5" t="n">
-        <v>0.04239028934904011</v>
+        <v>0.04239028934904009</v>
       </c>
       <c r="H5" t="n">
         <v>131.6527908126735</v>
       </c>
       <c r="I5" t="n">
-        <v>0.01129992791703305</v>
+        <v>0.01129992791703349</v>
       </c>
       <c r="J5" t="n">
-        <v>0.008576236258402314</v>
+        <v>0.008576236258402758</v>
       </c>
     </row>
     <row r="6">
@@ -1318,19 +1318,19 @@
         <v>302</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.2988165438463746</v>
+        <v>-0.2988165438463748</v>
       </c>
       <c r="G6" t="n">
-        <v>7.499254830416596e-35</v>
+        <v>7.499254830416286e-35</v>
       </c>
       <c r="H6" t="n">
-        <v>0.7124952190158385</v>
+        <v>0.7124952190158383</v>
       </c>
       <c r="I6" t="n">
-        <v>0.3973134761583396</v>
+        <v>0.3973134761583398</v>
       </c>
       <c r="J6" t="n">
-        <v>0.3953045210788673</v>
+        <v>0.3953045210788675</v>
       </c>
     </row>
     <row r="7">
@@ -1361,16 +1361,16 @@
         <v>-124.5232798972416</v>
       </c>
       <c r="G7" t="n">
-        <v>4.059895449149105e-21</v>
+        <v>4.059895449149172e-21</v>
       </c>
       <c r="H7" t="n">
         <v>130.1011388181451</v>
       </c>
       <c r="I7" t="n">
-        <v>0.2569298856856741</v>
+        <v>0.2569298856856742</v>
       </c>
       <c r="J7" t="n">
-        <v>0.2544529853046262</v>
+        <v>0.2544529853046263</v>
       </c>
     </row>
     <row r="8">
@@ -1401,16 +1401,16 @@
         <v>0.01403496035500879</v>
       </c>
       <c r="G8" t="n">
-        <v>0.00137200960855551</v>
+        <v>0.001372009608555512</v>
       </c>
       <c r="H8" t="n">
-        <v>0.6967623534130518</v>
+        <v>0.696762353413052</v>
       </c>
       <c r="I8" t="n">
-        <v>0.03548550672689432</v>
+        <v>0.03548550672689399</v>
       </c>
       <c r="J8" t="n">
-        <v>0.03208932893367911</v>
+        <v>0.03208932893367877</v>
       </c>
     </row>
     <row r="9">
@@ -1438,19 +1438,19 @@
         <v>286</v>
       </c>
       <c r="F9" t="n">
-        <v>6.791656856437388</v>
+        <v>6.791656856437389</v>
       </c>
       <c r="G9" t="n">
-        <v>0.01108464860441267</v>
+        <v>0.01108464860441266</v>
       </c>
       <c r="H9" t="n">
         <v>128.2026579529401</v>
       </c>
       <c r="I9" t="n">
-        <v>0.02250020147086329</v>
+        <v>0.02250020147086318</v>
       </c>
       <c r="J9" t="n">
-        <v>0.01905830077181692</v>
+        <v>0.01905830077181681</v>
       </c>
     </row>
     <row r="10">
@@ -1478,10 +1478,10 @@
         <v>256</v>
       </c>
       <c r="F10" t="n">
-        <v>0.007926639423187705</v>
+        <v>0.007926639423187767</v>
       </c>
       <c r="G10" t="n">
-        <v>0.01608804321031534</v>
+        <v>0.01608804321031447</v>
       </c>
       <c r="H10" t="n">
         <v>0.7007708363594571</v>
@@ -1518,19 +1518,19 @@
         <v>256</v>
       </c>
       <c r="F11" t="n">
-        <v>7.540815097683963</v>
+        <v>7.540815097683968</v>
       </c>
       <c r="G11" t="n">
-        <v>0.000255445445697456</v>
+        <v>0.0002554454456974526</v>
       </c>
       <c r="H11" t="n">
         <v>117.8771762474701</v>
       </c>
       <c r="I11" t="n">
-        <v>0.05138085831133465</v>
+        <v>0.05138085831133488</v>
       </c>
       <c r="J11" t="n">
-        <v>0.04764613728106437</v>
+        <v>0.04764613728106459</v>
       </c>
     </row>
   </sheetData>
@@ -1619,10 +1619,10 @@
         <v>524</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.002375311130268854</v>
+        <v>-0.002375311130268823</v>
       </c>
       <c r="G2" t="n">
-        <v>0.3452286286055533</v>
+        <v>0.3452286286055592</v>
       </c>
       <c r="H2" t="n">
         <v>0.7405879669180879</v>
@@ -1656,10 +1656,10 @@
         <v>524</v>
       </c>
       <c r="F3" t="n">
-        <v>-2.904173895654854</v>
+        <v>-2.904173895654835</v>
       </c>
       <c r="G3" t="n">
-        <v>0.02923977635331139</v>
+        <v>0.02923977635331236</v>
       </c>
       <c r="H3" t="n">
         <v>0.7451671756852611</v>
@@ -1693,10 +1693,10 @@
         <v>365</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.001897600882188976</v>
+        <v>-0.00189760088218894</v>
       </c>
       <c r="G4" t="n">
-        <v>0.3661624625650206</v>
+        <v>0.3661624625650293</v>
       </c>
       <c r="H4" t="n">
         <v>0.7157591781358699</v>
@@ -1730,10 +1730,10 @@
         <v>365</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.3919084267777011</v>
+        <v>-0.3919084267777631</v>
       </c>
       <c r="G5" t="n">
-        <v>0.6898257492991037</v>
+        <v>0.689825749299057</v>
       </c>
       <c r="H5" t="n">
         <v>0.7728342386974256</v>
@@ -1767,10 +1767,10 @@
         <v>302</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.09888435074694735</v>
+        <v>-0.09888435074694711</v>
       </c>
       <c r="G6" t="n">
-        <v>6.38649596433917e-05</v>
+        <v>6.386495964339403e-05</v>
       </c>
       <c r="H6" t="n">
         <v>0.6972015878915354</v>
@@ -1804,10 +1804,10 @@
         <v>302</v>
       </c>
       <c r="F7" t="n">
-        <v>-11.10004112186785</v>
+        <v>-11.10004112186764</v>
       </c>
       <c r="G7" t="n">
-        <v>0.3074964303100962</v>
+        <v>0.3074964303101052</v>
       </c>
       <c r="H7" t="n">
         <v>0.7762702692557996</v>
@@ -1841,10 +1841,10 @@
         <v>286</v>
       </c>
       <c r="F8" t="n">
-        <v>0.006010067131184558</v>
+        <v>0.00601006713118456</v>
       </c>
       <c r="G8" t="n">
-        <v>0.04119036045240992</v>
+        <v>0.04119036045241011</v>
       </c>
       <c r="H8" t="n">
         <v>0.5837877808931813</v>
@@ -1878,10 +1878,10 @@
         <v>286</v>
       </c>
       <c r="F9" t="n">
-        <v>1.529369551270922</v>
+        <v>1.529369551270992</v>
       </c>
       <c r="G9" t="n">
-        <v>0.3341571099737881</v>
+        <v>0.3341571099737659</v>
       </c>
       <c r="H9" t="n">
         <v>0.6719682038719668</v>
@@ -1915,16 +1915,16 @@
         <v>256</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.0005573381825121956</v>
+        <v>-0.0005573381825121296</v>
       </c>
       <c r="G10" t="n">
-        <v>0.8268690500638302</v>
+        <v>0.8268690500638504</v>
       </c>
       <c r="H10" t="n">
-        <v>0.4895939705541358</v>
+        <v>0.4895939705541357</v>
       </c>
       <c r="I10" t="n">
-        <v>0.4751873487552606</v>
+        <v>0.4751873487552605</v>
       </c>
     </row>
     <row r="11">
@@ -1952,16 +1952,16 @@
         <v>256</v>
       </c>
       <c r="F11" t="n">
-        <v>1.550535593455556</v>
+        <v>1.550535593455592</v>
       </c>
       <c r="G11" t="n">
-        <v>0.2514591870945995</v>
+        <v>0.2514591870945883</v>
       </c>
       <c r="H11" t="n">
-        <v>0.6398583379081237</v>
+        <v>0.6398583379081239</v>
       </c>
       <c r="I11" t="n">
-        <v>0.6296930490587562</v>
+        <v>0.6296930490587563</v>
       </c>
     </row>
   </sheetData>
@@ -1975,7 +1975,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K79"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2069,7 +2069,7 @@
         <v>-0.2181269853607984</v>
       </c>
       <c r="I2" t="n">
-        <v>1.636318146108423e-07</v>
+        <v>1.636318146108424e-07</v>
       </c>
       <c r="J2" t="n">
         <v>-0.1634106828747343</v>
@@ -2112,7 +2112,7 @@
         <v>0.05172034933756482</v>
       </c>
       <c r="I3" t="n">
-        <v>0.2196431099543466</v>
+        <v>0.2196431099543463</v>
       </c>
       <c r="J3" t="n">
         <v>0.03176276808162604</v>
@@ -2146,7 +2146,7 @@
         <v>565</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.443486750244555</v>
+        <v>-0.4434867502445549</v>
       </c>
       <c r="G4" t="n">
         <v>1.266446548651356e-28</v>
@@ -2155,7 +2155,7 @@
         <v>-0.5510468751917701</v>
       </c>
       <c r="I4" t="n">
-        <v>3.459841455205048e-46</v>
+        <v>3.459841455205077e-46</v>
       </c>
       <c r="J4" t="n">
         <v>-0.4056203749356901</v>
@@ -2189,7 +2189,7 @@
         <v>565</v>
       </c>
       <c r="F5" t="n">
-        <v>0.02014093814636463</v>
+        <v>0.02014093814636462</v>
       </c>
       <c r="G5" t="n">
         <v>0.6328403624859141</v>
@@ -2198,7 +2198,7 @@
         <v>0.01751911019795971</v>
       </c>
       <c r="I5" t="n">
-        <v>0.6777509176244131</v>
+        <v>0.6777509176244132</v>
       </c>
       <c r="J5" t="n">
         <v>0.01496932866156525</v>
@@ -2241,7 +2241,7 @@
         <v>-0.3311065516322187</v>
       </c>
       <c r="I6" t="n">
-        <v>6.373529467241609e-16</v>
+        <v>6.373529467241598e-16</v>
       </c>
       <c r="J6" t="n">
         <v>-0.2554772286084155</v>
@@ -2275,7 +2275,7 @@
         <v>524</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.06396633366734999</v>
+        <v>-0.06396633366734991</v>
       </c>
       <c r="G7" t="n">
         <v>0.143670717343492</v>
@@ -2284,7 +2284,7 @@
         <v>-0.1378035896698175</v>
       </c>
       <c r="I7" t="n">
-        <v>0.001566717372801578</v>
+        <v>0.001566717372801583</v>
       </c>
       <c r="J7" t="n">
         <v>-0.1094149914244232</v>
@@ -2364,13 +2364,13 @@
         <v>-0.4356149493069325</v>
       </c>
       <c r="G9" t="n">
-        <v>2.041725728456852e-15</v>
+        <v>2.041725728456778e-15</v>
       </c>
       <c r="H9" t="n">
         <v>-0.6272718864060146</v>
       </c>
       <c r="I9" t="n">
-        <v>1.955299293927514e-34</v>
+        <v>1.955299293927468e-34</v>
       </c>
       <c r="J9" t="n">
         <v>-0.4763504358110379</v>
@@ -2413,7 +2413,7 @@
         <v>0.1492268868940867</v>
       </c>
       <c r="I10" t="n">
-        <v>0.01151178507189819</v>
+        <v>0.0115117850718982</v>
       </c>
       <c r="J10" t="n">
         <v>0.1037599805501969</v>
@@ -2456,7 +2456,7 @@
         <v>0.1602234161541771</v>
       </c>
       <c r="I11" t="n">
-        <v>0.01023939208109393</v>
+        <v>0.01023939208109394</v>
       </c>
       <c r="J11" t="n">
         <v>0.1234214802651361</v>
@@ -2490,16 +2490,16 @@
         <v>565</v>
       </c>
       <c r="F12" t="n">
-        <v>0.7499678811548811</v>
+        <v>0.7499678811548812</v>
       </c>
       <c r="G12" t="n">
-        <v>3.97776710615413e-103</v>
+        <v>3.977767106153277e-103</v>
       </c>
       <c r="H12" t="n">
         <v>0.7795928516363934</v>
       </c>
       <c r="I12" t="n">
-        <v>1.649764303761214e-116</v>
+        <v>1.64976430376115e-116</v>
       </c>
       <c r="J12" t="n">
         <v>0.6032005594499876</v>
@@ -2533,16 +2533,16 @@
         <v>565</v>
       </c>
       <c r="F13" t="n">
-        <v>0.8173875628362024</v>
+        <v>0.8173875628362023</v>
       </c>
       <c r="G13" t="n">
-        <v>5.874407466438861e-137</v>
+        <v>5.874407466440671e-137</v>
       </c>
       <c r="H13" t="n">
         <v>0.8206801592553979</v>
       </c>
       <c r="I13" t="n">
-        <v>5.809000361350459e-139</v>
+        <v>5.809000361350647e-139</v>
       </c>
       <c r="J13" t="n">
         <v>0.6551802113587517</v>
@@ -2554,44 +2554,44 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>d002_nm</t>
+          <t>carbonization_temperature_C</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>d002</t>
+          <t>Carbonization temperature</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>id_ig</t>
+          <t>reversible_capacity_mAh_g</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>ID/IG</t>
+          <t>Reversible capacity</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>565</v>
+        <v>558</v>
       </c>
       <c r="F14" t="n">
-        <v>0.1423338000578228</v>
+        <v>0.1995204821513981</v>
       </c>
       <c r="G14" t="n">
-        <v>0.0006912327370564002</v>
+        <v>2.030620807237947e-06</v>
       </c>
       <c r="H14" t="n">
-        <v>0.1820492659745402</v>
+        <v>0.2560156529428892</v>
       </c>
       <c r="I14" t="n">
-        <v>1.336057467872995e-05</v>
+        <v>8.430153510948003e-10</v>
       </c>
       <c r="J14" t="n">
-        <v>0.1284426252988861</v>
+        <v>0.1874713574210626</v>
       </c>
       <c r="K14" t="n">
-        <v>6.319280025555388e-06</v>
+        <v>2.463310652219405e-10</v>
       </c>
     </row>
     <row r="15">
@@ -2607,34 +2607,34 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ssa_m2_g</t>
+          <t>id_ig</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>SSA</t>
+          <t>ID/IG</t>
         </is>
       </c>
       <c r="E15" t="n">
         <v>565</v>
       </c>
       <c r="F15" t="n">
-        <v>0.100410463871457</v>
+        <v>0.1423338000578228</v>
       </c>
       <c r="G15" t="n">
-        <v>0.01696431621020364</v>
+        <v>0.0006912327370564002</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1493305530306386</v>
+        <v>0.1820492659745402</v>
       </c>
       <c r="I15" t="n">
-        <v>0.0003684957964075374</v>
+        <v>1.336057467872996e-05</v>
       </c>
       <c r="J15" t="n">
-        <v>0.101100790681851</v>
+        <v>0.1284426252988861</v>
       </c>
       <c r="K15" t="n">
-        <v>0.0003690252118780625</v>
+        <v>6.319280025555388e-06</v>
       </c>
     </row>
     <row r="16">
@@ -2650,34 +2650,34 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>electrolyte_type</t>
+          <t>ssa_m2_g</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Electrolyte type</t>
+          <t>SSA</t>
         </is>
       </c>
       <c r="E16" t="n">
         <v>565</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.02441064951730194</v>
+        <v>0.100410463871457</v>
       </c>
       <c r="G16" t="n">
-        <v>0.5625650251989687</v>
+        <v>0.01696431621020364</v>
       </c>
       <c r="H16" t="n">
-        <v>-0.01842970173689641</v>
+        <v>0.1493305530306386</v>
       </c>
       <c r="I16" t="n">
-        <v>0.6620127424475525</v>
+        <v>0.0003684957964075375</v>
       </c>
       <c r="J16" t="n">
-        <v>-0.01519412256189604</v>
+        <v>0.101100790681851</v>
       </c>
       <c r="K16" t="n">
-        <v>0.6616174242488522</v>
+        <v>0.0003690252118780625</v>
       </c>
     </row>
     <row r="17">
@@ -2693,34 +2693,34 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>current_density_mA_g</t>
+          <t>electrolyte_type</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Current density</t>
+          <t>Electrolyte type</t>
         </is>
       </c>
       <c r="E17" t="n">
         <v>565</v>
       </c>
       <c r="F17" t="n">
-        <v>-0.0007626572240376425</v>
+        <v>-0.02441064951730194</v>
       </c>
       <c r="G17" t="n">
-        <v>0.9855686426487615</v>
+        <v>0.5625650251989687</v>
       </c>
       <c r="H17" t="n">
-        <v>0.07982990348957315</v>
+        <v>-0.01842970173689641</v>
       </c>
       <c r="I17" t="n">
-        <v>0.05791243780797913</v>
+        <v>0.6620127424475525</v>
       </c>
       <c r="J17" t="n">
-        <v>0.05918815671208932</v>
+        <v>-0.01519412256189604</v>
       </c>
       <c r="K17" t="n">
-        <v>0.05485779293764693</v>
+        <v>0.6616174242488522</v>
       </c>
     </row>
     <row r="18">
@@ -2736,34 +2736,34 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>carbonization_time_h</t>
+          <t>current_density_mA_g</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Carbonization time</t>
+          <t>Current density</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>524</v>
+        <v>565</v>
       </c>
       <c r="F18" t="n">
-        <v>-0.0144382863433448</v>
+        <v>-0.0007626572240376209</v>
       </c>
       <c r="G18" t="n">
-        <v>0.7415999195573121</v>
+        <v>0.9855686426487615</v>
       </c>
       <c r="H18" t="n">
-        <v>0.04798388613797423</v>
+        <v>0.07982990348957315</v>
       </c>
       <c r="I18" t="n">
-        <v>0.2728994427506401</v>
+        <v>0.05791243780797913</v>
       </c>
       <c r="J18" t="n">
-        <v>0.03675852808342851</v>
+        <v>0.05918815671208932</v>
       </c>
       <c r="K18" t="n">
-        <v>0.2732203665482589</v>
+        <v>0.05485779293764693</v>
       </c>
     </row>
     <row r="19">
@@ -2779,34 +2779,34 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>heating_rate_C_min</t>
+          <t>carbonization_time_h</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Heating rate</t>
+          <t>Carbonization time</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>365</v>
+        <v>524</v>
       </c>
       <c r="F19" t="n">
-        <v>-0.00794212712792541</v>
+        <v>-0.01443828634334479</v>
       </c>
       <c r="G19" t="n">
-        <v>0.8798052877994758</v>
+        <v>0.7415999195573121</v>
       </c>
       <c r="H19" t="n">
-        <v>-0.008980922837386416</v>
+        <v>0.04798388613797423</v>
       </c>
       <c r="I19" t="n">
-        <v>0.8642275345738918</v>
+        <v>0.2728994427506399</v>
       </c>
       <c r="J19" t="n">
-        <v>-0.006398840720646511</v>
+        <v>0.03675852808342851</v>
       </c>
       <c r="K19" t="n">
-        <v>0.873945672734375</v>
+        <v>0.2732203665482589</v>
       </c>
     </row>
     <row r="20">
@@ -2822,34 +2822,34 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>pore_volume_cm3_g</t>
+          <t>heating_rate_C_min</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Pore volume</t>
+          <t>Heating rate</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>302</v>
+        <v>365</v>
       </c>
       <c r="F20" t="n">
-        <v>0.06606399418503518</v>
+        <v>-0.007942127127925427</v>
       </c>
       <c r="G20" t="n">
-        <v>0.252391645238652</v>
+        <v>0.8798052877994758</v>
       </c>
       <c r="H20" t="n">
-        <v>0.134916825756546</v>
+        <v>-0.008980922837386416</v>
       </c>
       <c r="I20" t="n">
-        <v>0.01899568257757459</v>
+        <v>0.8642275345738917</v>
       </c>
       <c r="J20" t="n">
-        <v>0.09187204775424389</v>
+        <v>-0.006398840720646511</v>
       </c>
       <c r="K20" t="n">
-        <v>0.01855569201628276</v>
+        <v>0.873945672734375</v>
       </c>
     </row>
     <row r="21">
@@ -2865,34 +2865,34 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>lc_nm</t>
+          <t>pore_volume_cm3_g</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Lc</t>
+          <t>Pore volume</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>286</v>
+        <v>302</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.03768649236385627</v>
+        <v>0.0660639941850352</v>
       </c>
       <c r="G21" t="n">
-        <v>0.525577922337002</v>
+        <v>0.252391645238652</v>
       </c>
       <c r="H21" t="n">
-        <v>-0.1314004530187621</v>
+        <v>0.134916825756546</v>
       </c>
       <c r="I21" t="n">
-        <v>0.02627690886000911</v>
+        <v>0.01899568257757462</v>
       </c>
       <c r="J21" t="n">
-        <v>-0.09082887547153634</v>
+        <v>0.09187204775424389</v>
       </c>
       <c r="K21" t="n">
-        <v>0.02346564393162545</v>
+        <v>0.01855569201628276</v>
       </c>
     </row>
     <row r="22">
@@ -2908,34 +2908,34 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>la_nm</t>
+          <t>lc_nm</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>La</t>
+          <t>Lc</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>256</v>
+        <v>286</v>
       </c>
       <c r="F22" t="n">
-        <v>0.01465862707216834</v>
+        <v>-0.03768649236385626</v>
       </c>
       <c r="G22" t="n">
-        <v>0.8154486482202745</v>
+        <v>0.525577922337002</v>
       </c>
       <c r="H22" t="n">
-        <v>0.005787969049062654</v>
+        <v>-0.1314004530187621</v>
       </c>
       <c r="I22" t="n">
-        <v>0.9265748334254018</v>
+        <v>0.02627690886000911</v>
       </c>
       <c r="J22" t="n">
-        <v>0.001483885259921387</v>
+        <v>-0.09082887547153634</v>
       </c>
       <c r="K22" t="n">
-        <v>0.9720270631316147</v>
+        <v>0.02346564393162545</v>
       </c>
     </row>
     <row r="23">
@@ -2951,34 +2951,34 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ice</t>
+          <t>la_nm</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>La</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>565</v>
+        <v>256</v>
       </c>
       <c r="F23" t="n">
-        <v>-0.1255910021135957</v>
+        <v>0.01465862707216833</v>
       </c>
       <c r="G23" t="n">
-        <v>0.002785196898588286</v>
+        <v>0.8154486482202745</v>
       </c>
       <c r="H23" t="n">
-        <v>-0.09558218870958307</v>
+        <v>0.005787969049062654</v>
       </c>
       <c r="I23" t="n">
-        <v>0.02307833981243183</v>
+        <v>0.9265748334254018</v>
       </c>
       <c r="J23" t="n">
-        <v>-0.06634409354020061</v>
+        <v>0.001483885259921387</v>
       </c>
       <c r="K23" t="n">
-        <v>0.01954965197626471</v>
+        <v>0.9720270631316147</v>
       </c>
     </row>
     <row r="24">
@@ -2994,120 +2994,120 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>plateau_capacity_mAh_g</t>
+          <t>ice</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Plateau capacity</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="E24" t="n">
         <v>565</v>
       </c>
       <c r="F24" t="n">
-        <v>-0.07225381674120777</v>
+        <v>-0.1255910021135957</v>
       </c>
       <c r="G24" t="n">
-        <v>0.08618156891629511</v>
+        <v>0.002785196898588286</v>
       </c>
       <c r="H24" t="n">
-        <v>-0.0440993365854058</v>
+        <v>-0.09558218870958307</v>
       </c>
       <c r="I24" t="n">
-        <v>0.2953685805416671</v>
+        <v>0.02307833981243183</v>
       </c>
       <c r="J24" t="n">
-        <v>-0.03277189678641169</v>
+        <v>-0.06634409354020061</v>
       </c>
       <c r="K24" t="n">
-        <v>0.25582738107283</v>
+        <v>0.01954965197626471</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>id_ig</t>
+          <t>d002_nm</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ID/IG</t>
+          <t>d002</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ssa_m2_g</t>
+          <t>plateau_capacity_mAh_g</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>SSA</t>
+          <t>Plateau capacity</t>
         </is>
       </c>
       <c r="E25" t="n">
         <v>565</v>
       </c>
       <c r="F25" t="n">
-        <v>-0.003669511553609553</v>
+        <v>-0.07225381674120779</v>
       </c>
       <c r="G25" t="n">
-        <v>0.9306473335406905</v>
+        <v>0.08618156891629414</v>
       </c>
       <c r="H25" t="n">
-        <v>-0.05870898066704883</v>
+        <v>-0.0440993365854058</v>
       </c>
       <c r="I25" t="n">
-        <v>0.1634359356975874</v>
+        <v>0.2953685805416666</v>
       </c>
       <c r="J25" t="n">
-        <v>-0.03881652088300067</v>
+        <v>-0.03277189678641169</v>
       </c>
       <c r="K25" t="n">
-        <v>0.1687368176320793</v>
+        <v>0.25582738107283</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>id_ig</t>
+          <t>d002_nm</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ID/IG</t>
+          <t>d002</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>electrolyte_type</t>
+          <t>reversible_capacity_mAh_g</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Electrolyte type</t>
+          <t>Reversible capacity</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>565</v>
+        <v>558</v>
       </c>
       <c r="F26" t="n">
-        <v>-0.03023489676637762</v>
+        <v>0.06833061392295256</v>
       </c>
       <c r="G26" t="n">
-        <v>0.473221291998826</v>
+        <v>0.1068808542643762</v>
       </c>
       <c r="H26" t="n">
-        <v>-0.02927023884847913</v>
+        <v>0.09285856430733569</v>
       </c>
       <c r="I26" t="n">
-        <v>0.4874604936253757</v>
+        <v>0.02828367468378303</v>
       </c>
       <c r="J26" t="n">
-        <v>-0.02397406592813114</v>
+        <v>0.06430010111061572</v>
       </c>
       <c r="K26" t="n">
-        <v>0.486974049825118</v>
+        <v>0.02443638182744086</v>
       </c>
     </row>
     <row r="27">
@@ -3123,34 +3123,34 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>current_density_mA_g</t>
+          <t>ssa_m2_g</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Current density</t>
+          <t>SSA</t>
         </is>
       </c>
       <c r="E27" t="n">
         <v>565</v>
       </c>
       <c r="F27" t="n">
-        <v>-0.1019034942642348</v>
+        <v>-0.003669511553609557</v>
       </c>
       <c r="G27" t="n">
-        <v>0.0153859417694675</v>
+        <v>0.9306473335406905</v>
       </c>
       <c r="H27" t="n">
-        <v>-0.123733417636351</v>
+        <v>-0.05870898066704883</v>
       </c>
       <c r="I27" t="n">
-        <v>0.003219913110042519</v>
+        <v>0.1634359356975873</v>
       </c>
       <c r="J27" t="n">
-        <v>-0.08960145817612446</v>
+        <v>-0.03881652088300067</v>
       </c>
       <c r="K27" t="n">
-        <v>0.003437583620322431</v>
+        <v>0.1687368176320793</v>
       </c>
     </row>
     <row r="28">
@@ -3166,34 +3166,34 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>carbonization_time_h</t>
+          <t>electrolyte_type</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Carbonization time</t>
+          <t>Electrolyte type</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>524</v>
+        <v>565</v>
       </c>
       <c r="F28" t="n">
-        <v>-0.02340331474766981</v>
+        <v>-0.0302348967663776</v>
       </c>
       <c r="G28" t="n">
-        <v>0.592981679480803</v>
+        <v>0.473221291998826</v>
       </c>
       <c r="H28" t="n">
-        <v>-0.00185000449341969</v>
+        <v>-0.02927023884847913</v>
       </c>
       <c r="I28" t="n">
-        <v>0.9663014436174344</v>
+        <v>0.4874604936253757</v>
       </c>
       <c r="J28" t="n">
-        <v>-0.002344202550249296</v>
+        <v>-0.02397406592813114</v>
       </c>
       <c r="K28" t="n">
-        <v>0.9439222360126152</v>
+        <v>0.486974049825118</v>
       </c>
     </row>
     <row r="29">
@@ -3209,34 +3209,34 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>heating_rate_C_min</t>
+          <t>current_density_mA_g</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Heating rate</t>
+          <t>Current density</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>365</v>
+        <v>565</v>
       </c>
       <c r="F29" t="n">
-        <v>0.04477283400316443</v>
+        <v>-0.1019034942642348</v>
       </c>
       <c r="G29" t="n">
-        <v>0.3937272194367734</v>
+        <v>0.0153859417694675</v>
       </c>
       <c r="H29" t="n">
-        <v>0.05775571868068568</v>
+        <v>-0.123733417636351</v>
       </c>
       <c r="I29" t="n">
-        <v>0.2710901453410258</v>
+        <v>0.003219913110042526</v>
       </c>
       <c r="J29" t="n">
-        <v>0.04573817511657489</v>
+        <v>-0.08960145817612446</v>
       </c>
       <c r="K29" t="n">
-        <v>0.2535915036019953</v>
+        <v>0.003437583620322431</v>
       </c>
     </row>
     <row r="30">
@@ -3252,34 +3252,34 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>pore_volume_cm3_g</t>
+          <t>carbonization_time_h</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Pore volume</t>
+          <t>Carbonization time</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>302</v>
+        <v>524</v>
       </c>
       <c r="F30" t="n">
-        <v>-0.1041130705708858</v>
+        <v>-0.0234033147476698</v>
       </c>
       <c r="G30" t="n">
-        <v>0.07080874763282673</v>
+        <v>0.592981679480803</v>
       </c>
       <c r="H30" t="n">
-        <v>-0.079560980663301</v>
+        <v>-0.00185000449341969</v>
       </c>
       <c r="I30" t="n">
-        <v>0.1678714010495902</v>
+        <v>0.9663014436174344</v>
       </c>
       <c r="J30" t="n">
-        <v>-0.05275546770428205</v>
+        <v>-0.002344202550249296</v>
       </c>
       <c r="K30" t="n">
-        <v>0.1734310161605681</v>
+        <v>0.9439222360126152</v>
       </c>
     </row>
     <row r="31">
@@ -3295,34 +3295,34 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>lc_nm</t>
+          <t>heating_rate_C_min</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Lc</t>
+          <t>Heating rate</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>286</v>
+        <v>365</v>
       </c>
       <c r="F31" t="n">
-        <v>0.01124163684768274</v>
+        <v>0.04477283400316443</v>
       </c>
       <c r="G31" t="n">
-        <v>0.8498681027763104</v>
+        <v>0.3937272194367734</v>
       </c>
       <c r="H31" t="n">
-        <v>-0.02999066206503953</v>
+        <v>0.05775571868068568</v>
       </c>
       <c r="I31" t="n">
-        <v>0.6135022628611301</v>
+        <v>0.2710901453410259</v>
       </c>
       <c r="J31" t="n">
-        <v>-0.01756741784540412</v>
+        <v>0.04573817511657489</v>
       </c>
       <c r="K31" t="n">
-        <v>0.6591142464302993</v>
+        <v>0.2535915036019953</v>
       </c>
     </row>
     <row r="32">
@@ -3338,34 +3338,34 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>la_nm</t>
+          <t>pore_volume_cm3_g</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>La</t>
+          <t>Pore volume</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>256</v>
+        <v>302</v>
       </c>
       <c r="F32" t="n">
-        <v>0.07075660825308508</v>
+        <v>-0.1041130705708858</v>
       </c>
       <c r="G32" t="n">
-        <v>0.259328473656788</v>
+        <v>0.07080874763282673</v>
       </c>
       <c r="H32" t="n">
-        <v>0.04840502246995132</v>
+        <v>-0.079560980663301</v>
       </c>
       <c r="I32" t="n">
-        <v>0.4406225595498851</v>
+        <v>0.1678714010495903</v>
       </c>
       <c r="J32" t="n">
-        <v>0.03117564020481876</v>
+        <v>-0.05275546770428205</v>
       </c>
       <c r="K32" t="n">
-        <v>0.4585142024383978</v>
+        <v>0.1734310161605681</v>
       </c>
     </row>
     <row r="33">
@@ -3381,34 +3381,34 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ice</t>
+          <t>lc_nm</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>Lc</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>565</v>
+        <v>286</v>
       </c>
       <c r="F33" t="n">
-        <v>0.06843298811784779</v>
+        <v>0.01124163684768275</v>
       </c>
       <c r="G33" t="n">
-        <v>0.1041760997424921</v>
+        <v>0.8498681027763104</v>
       </c>
       <c r="H33" t="n">
-        <v>0.1386432487735146</v>
+        <v>-0.02999066206503953</v>
       </c>
       <c r="I33" t="n">
-        <v>0.0009525310842178509</v>
+        <v>0.6135022628611302</v>
       </c>
       <c r="J33" t="n">
-        <v>0.09235939217904243</v>
+        <v>-0.01756741784540412</v>
       </c>
       <c r="K33" t="n">
-        <v>0.001068900122913918</v>
+        <v>0.6591142464302993</v>
       </c>
     </row>
     <row r="34">
@@ -3424,163 +3424,163 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>plateau_capacity_mAh_g</t>
+          <t>la_nm</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Plateau capacity</t>
+          <t>La</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>565</v>
+        <v>256</v>
       </c>
       <c r="F34" t="n">
-        <v>0.05287409906917159</v>
+        <v>0.07075660825308507</v>
       </c>
       <c r="G34" t="n">
-        <v>0.2095159603799352</v>
+        <v>0.259328473656788</v>
       </c>
       <c r="H34" t="n">
-        <v>0.1365397438371289</v>
+        <v>0.04840502246995132</v>
       </c>
       <c r="I34" t="n">
-        <v>0.001139627458461307</v>
+        <v>0.440622559549885</v>
       </c>
       <c r="J34" t="n">
-        <v>0.09276697369342404</v>
+        <v>0.03117564020481876</v>
       </c>
       <c r="K34" t="n">
-        <v>0.001205392836867296</v>
+        <v>0.4585142024383978</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ssa_m2_g</t>
+          <t>id_ig</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>SSA</t>
+          <t>ID/IG</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>electrolyte_type</t>
+          <t>ice</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Electrolyte type</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="E35" t="n">
         <v>565</v>
       </c>
       <c r="F35" t="n">
-        <v>0.01578769580411299</v>
+        <v>0.06843298811784779</v>
       </c>
       <c r="G35" t="n">
-        <v>0.7080609980044772</v>
+        <v>0.1041760997424921</v>
       </c>
       <c r="H35" t="n">
-        <v>0.0507838194422963</v>
+        <v>0.1386432487735146</v>
       </c>
       <c r="I35" t="n">
-        <v>0.2281175972529115</v>
+        <v>0.0009525310842178511</v>
       </c>
       <c r="J35" t="n">
-        <v>0.04151196779495249</v>
+        <v>0.09235939217904243</v>
       </c>
       <c r="K35" t="n">
-        <v>0.2277986403833989</v>
+        <v>0.001068900122913918</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ssa_m2_g</t>
+          <t>id_ig</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>SSA</t>
+          <t>ID/IG</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>current_density_mA_g</t>
+          <t>plateau_capacity_mAh_g</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Current density</t>
+          <t>Plateau capacity</t>
         </is>
       </c>
       <c r="E36" t="n">
         <v>565</v>
       </c>
       <c r="F36" t="n">
-        <v>0.343706216447519</v>
+        <v>0.0528740990691716</v>
       </c>
       <c r="G36" t="n">
-        <v>4.126499645843004e-17</v>
+        <v>0.2095159603799352</v>
       </c>
       <c r="H36" t="n">
-        <v>0.2965407630860846</v>
+        <v>0.1365397438371289</v>
       </c>
       <c r="I36" t="n">
-        <v>6.220717267837881e-13</v>
+        <v>0.001139627458461307</v>
       </c>
       <c r="J36" t="n">
-        <v>0.21316360116485</v>
+        <v>0.09276697369342404</v>
       </c>
       <c r="K36" t="n">
-        <v>3.079901696240681e-12</v>
+        <v>0.001205392836867296</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ssa_m2_g</t>
+          <t>id_ig</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>SSA</t>
+          <t>ID/IG</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>carbonization_time_h</t>
+          <t>reversible_capacity_mAh_g</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Carbonization time</t>
+          <t>Reversible capacity</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>524</v>
+        <v>558</v>
       </c>
       <c r="F37" t="n">
-        <v>0.008944167085313762</v>
+        <v>-0.08927954845356463</v>
       </c>
       <c r="G37" t="n">
-        <v>0.8381530754896541</v>
+        <v>0.03499240255627823</v>
       </c>
       <c r="H37" t="n">
-        <v>0.05970077179194353</v>
+        <v>-0.04747899444593579</v>
       </c>
       <c r="I37" t="n">
-        <v>0.172389230554131</v>
+        <v>0.2628559418076807</v>
       </c>
       <c r="J37" t="n">
-        <v>0.0451490561681537</v>
+        <v>-0.03031559061572308</v>
       </c>
       <c r="K37" t="n">
-        <v>0.1746444681428926</v>
+        <v>0.2855787073041423</v>
       </c>
     </row>
     <row r="38">
@@ -3596,34 +3596,34 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>heating_rate_C_min</t>
+          <t>electrolyte_type</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Heating rate</t>
+          <t>Electrolyte type</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>365</v>
+        <v>565</v>
       </c>
       <c r="F38" t="n">
-        <v>0.03216675496613058</v>
+        <v>0.01578769580411298</v>
       </c>
       <c r="G38" t="n">
-        <v>0.5401437635461958</v>
+        <v>0.7080609980044772</v>
       </c>
       <c r="H38" t="n">
-        <v>0.05437419989054413</v>
+        <v>0.0507838194422963</v>
       </c>
       <c r="I38" t="n">
-        <v>0.3001923381796873</v>
+        <v>0.2281175972529114</v>
       </c>
       <c r="J38" t="n">
-        <v>0.04215283149776887</v>
+        <v>0.04151196779495249</v>
       </c>
       <c r="K38" t="n">
-        <v>0.2918307622178755</v>
+        <v>0.2277986403833989</v>
       </c>
     </row>
     <row r="39">
@@ -3639,34 +3639,34 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>pore_volume_cm3_g</t>
+          <t>current_density_mA_g</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Pore volume</t>
+          <t>Current density</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>302</v>
+        <v>565</v>
       </c>
       <c r="F39" t="n">
-        <v>0.7631740185041012</v>
+        <v>0.343706216447519</v>
       </c>
       <c r="G39" t="n">
-        <v>7.72765060227087e-59</v>
+        <v>4.126499645843004e-17</v>
       </c>
       <c r="H39" t="n">
-        <v>0.8859688582065801</v>
+        <v>0.2965407630860846</v>
       </c>
       <c r="I39" t="n">
-        <v>3.971041921907264e-102</v>
+        <v>6.220717267837881e-13</v>
       </c>
       <c r="J39" t="n">
-        <v>0.7071300237700989</v>
+        <v>0.21316360116485</v>
       </c>
       <c r="K39" t="n">
-        <v>1.043782717534748e-74</v>
+        <v>3.079901696240681e-12</v>
       </c>
     </row>
     <row r="40">
@@ -3682,34 +3682,34 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>lc_nm</t>
+          <t>carbonization_time_h</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Lc</t>
+          <t>Carbonization time</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>286</v>
+        <v>524</v>
       </c>
       <c r="F40" t="n">
-        <v>-0.1075636872097107</v>
+        <v>0.008944167085313766</v>
       </c>
       <c r="G40" t="n">
-        <v>0.06931306279252639</v>
+        <v>0.8381530754896541</v>
       </c>
       <c r="H40" t="n">
-        <v>-0.08435674252058659</v>
+        <v>0.05970077179194353</v>
       </c>
       <c r="I40" t="n">
-        <v>0.1547675820105515</v>
+        <v>0.172389230554131</v>
       </c>
       <c r="J40" t="n">
-        <v>-0.05600521126092554</v>
+        <v>0.0451490561681537</v>
       </c>
       <c r="K40" t="n">
-        <v>0.1589136485598043</v>
+        <v>0.1746444681428926</v>
       </c>
     </row>
     <row r="41">
@@ -3725,34 +3725,34 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>la_nm</t>
+          <t>heating_rate_C_min</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>La</t>
+          <t>Heating rate</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>256</v>
+        <v>365</v>
       </c>
       <c r="F41" t="n">
-        <v>-0.1936229624456837</v>
+        <v>0.03216675496613057</v>
       </c>
       <c r="G41" t="n">
-        <v>0.001856283747681796</v>
+        <v>0.5401437635461958</v>
       </c>
       <c r="H41" t="n">
-        <v>-0.2192378910459487</v>
+        <v>0.05437419989054413</v>
       </c>
       <c r="I41" t="n">
-        <v>0.0004097436248579172</v>
+        <v>0.3001923381796873</v>
       </c>
       <c r="J41" t="n">
-        <v>-0.1414925146581904</v>
+        <v>0.04215283149776887</v>
       </c>
       <c r="K41" t="n">
-        <v>0.0007525980071549126</v>
+        <v>0.2918307622178755</v>
       </c>
     </row>
     <row r="42">
@@ -3768,34 +3768,34 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ice</t>
+          <t>pore_volume_cm3_g</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>Pore volume</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>565</v>
+        <v>302</v>
       </c>
       <c r="F42" t="n">
-        <v>-0.646111534598435</v>
+        <v>0.7631740185041009</v>
       </c>
       <c r="G42" t="n">
-        <v>4.511222956921875e-68</v>
+        <v>7.727650602271812e-59</v>
       </c>
       <c r="H42" t="n">
-        <v>-0.6836086929694647</v>
+        <v>0.8859688582065801</v>
       </c>
       <c r="I42" t="n">
-        <v>4.908047533621369e-79</v>
+        <v>3.971041921907224e-102</v>
       </c>
       <c r="J42" t="n">
-        <v>-0.5057590414293713</v>
+        <v>0.7071300237700989</v>
       </c>
       <c r="K42" t="n">
-        <v>4.653597704901204e-72</v>
+        <v>1.043782717534748e-74</v>
       </c>
     </row>
     <row r="43">
@@ -3811,206 +3811,206 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>plateau_capacity_mAh_g</t>
+          <t>lc_nm</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Plateau capacity</t>
+          <t>Lc</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>565</v>
+        <v>286</v>
       </c>
       <c r="F43" t="n">
-        <v>-0.5295537533936092</v>
+        <v>-0.1075636872097107</v>
       </c>
       <c r="G43" t="n">
-        <v>3.691263880872587e-42</v>
+        <v>0.06931306279252639</v>
       </c>
       <c r="H43" t="n">
-        <v>-0.6247816345029006</v>
+        <v>-0.08435674252058659</v>
       </c>
       <c r="I43" t="n">
-        <v>1.695648750418406e-62</v>
+        <v>0.1547675820105515</v>
       </c>
       <c r="J43" t="n">
-        <v>-0.4544369390647887</v>
+        <v>-0.05600521126092554</v>
       </c>
       <c r="K43" t="n">
-        <v>7.239808688259662e-57</v>
+        <v>0.1589136485598043</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>electrolyte_type</t>
+          <t>ssa_m2_g</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Electrolyte type</t>
+          <t>SSA</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>current_density_mA_g</t>
+          <t>la_nm</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Current density</t>
+          <t>La</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>565</v>
+        <v>256</v>
       </c>
       <c r="F44" t="n">
-        <v>0.05950044929577328</v>
+        <v>-0.1936229624456837</v>
       </c>
       <c r="G44" t="n">
-        <v>0.1578237043438263</v>
+        <v>0.001856283747681796</v>
       </c>
       <c r="H44" t="n">
-        <v>0.1094138764239998</v>
+        <v>-0.2192378910459487</v>
       </c>
       <c r="I44" t="n">
-        <v>0.009246675331718255</v>
+        <v>0.0004097436248579178</v>
       </c>
       <c r="J44" t="n">
-        <v>0.09713827205002599</v>
+        <v>-0.1414925146581904</v>
       </c>
       <c r="K44" t="n">
-        <v>0.009364961095298347</v>
+        <v>0.0007525980071549126</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>electrolyte_type</t>
+          <t>ssa_m2_g</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Electrolyte type</t>
+          <t>SSA</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>carbonization_time_h</t>
+          <t>ice</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Carbonization time</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>524</v>
+        <v>565</v>
       </c>
       <c r="F45" t="n">
-        <v>0.02460402072018155</v>
+        <v>-0.6461115345984351</v>
       </c>
       <c r="G45" t="n">
-        <v>0.574148836042561</v>
+        <v>4.511222956921249e-68</v>
       </c>
       <c r="H45" t="n">
-        <v>0.1102105775573811</v>
+        <v>-0.6836086929694647</v>
       </c>
       <c r="I45" t="n">
-        <v>0.01158613371795066</v>
+        <v>4.908047533621248e-79</v>
       </c>
       <c r="J45" t="n">
-        <v>0.1025301495602896</v>
+        <v>-0.5057590414293713</v>
       </c>
       <c r="K45" t="n">
-        <v>0.01172125493550799</v>
+        <v>4.653597704901204e-72</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>electrolyte_type</t>
+          <t>ssa_m2_g</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Electrolyte type</t>
+          <t>SSA</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>heating_rate_C_min</t>
+          <t>plateau_capacity_mAh_g</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Heating rate</t>
+          <t>Plateau capacity</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>365</v>
+        <v>565</v>
       </c>
       <c r="F46" t="n">
-        <v>0.01629854084767969</v>
+        <v>-0.5295537533936093</v>
       </c>
       <c r="G46" t="n">
-        <v>0.7563056581858302</v>
+        <v>3.691263880872587e-42</v>
       </c>
       <c r="H46" t="n">
-        <v>0.0123581641819504</v>
+        <v>-0.6247816345029006</v>
       </c>
       <c r="I46" t="n">
-        <v>0.8139747042176797</v>
+        <v>1.695648750418408e-62</v>
       </c>
       <c r="J46" t="n">
-        <v>0.01152656901910095</v>
+        <v>-0.4544369390647887</v>
       </c>
       <c r="K46" t="n">
-        <v>0.8136043619314126</v>
+        <v>7.239808688259662e-57</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>electrolyte_type</t>
+          <t>ssa_m2_g</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Electrolyte type</t>
+          <t>SSA</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>pore_volume_cm3_g</t>
+          <t>reversible_capacity_mAh_g</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Pore volume</t>
+          <t>Reversible capacity</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>302</v>
+        <v>558</v>
       </c>
       <c r="F47" t="n">
-        <v>-0.07074629617880274</v>
+        <v>-0.03846128090225396</v>
       </c>
       <c r="G47" t="n">
-        <v>0.2202447204383185</v>
+        <v>0.3644959108242139</v>
       </c>
       <c r="H47" t="n">
-        <v>-0.09180477632184833</v>
+        <v>-0.1975504284033616</v>
       </c>
       <c r="I47" t="n">
-        <v>0.1113521838275142</v>
+        <v>2.56999148310704e-06</v>
       </c>
       <c r="J47" t="n">
-        <v>-0.075230627298839</v>
+        <v>-0.140493238519178</v>
       </c>
       <c r="K47" t="n">
-        <v>0.1112155362240629</v>
+        <v>7.096761420722806e-07</v>
       </c>
     </row>
     <row r="48">
@@ -4026,34 +4026,34 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>lc_nm</t>
+          <t>current_density_mA_g</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Lc</t>
+          <t>Current density</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>286</v>
+        <v>565</v>
       </c>
       <c r="F48" t="n">
-        <v>-0.09781715798135987</v>
+        <v>0.05950044929577317</v>
       </c>
       <c r="G48" t="n">
-        <v>0.09874776382654843</v>
+        <v>0.1578237043438278</v>
       </c>
       <c r="H48" t="n">
-        <v>-0.1641349420705074</v>
+        <v>0.1094138764239998</v>
       </c>
       <c r="I48" t="n">
-        <v>0.005393974357511183</v>
+        <v>0.009246675331718256</v>
       </c>
       <c r="J48" t="n">
-        <v>-0.1345304650379796</v>
+        <v>0.09713827205002599</v>
       </c>
       <c r="K48" t="n">
-        <v>0.005589871837256947</v>
+        <v>0.009364961095298347</v>
       </c>
     </row>
     <row r="49">
@@ -4069,34 +4069,34 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>la_nm</t>
+          <t>carbonization_time_h</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>La</t>
+          <t>Carbonization time</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>256</v>
+        <v>524</v>
       </c>
       <c r="F49" t="n">
-        <v>-0.2283888372891541</v>
+        <v>0.02460402072018146</v>
       </c>
       <c r="G49" t="n">
-        <v>0.0002285568410490067</v>
+        <v>0.5741488360425644</v>
       </c>
       <c r="H49" t="n">
-        <v>-0.3008459514899685</v>
+        <v>0.1102105775573811</v>
       </c>
       <c r="I49" t="n">
-        <v>9.387539543675832e-07</v>
+        <v>0.01158613371795066</v>
       </c>
       <c r="J49" t="n">
-        <v>-0.2462639562527961</v>
+        <v>0.1025301495602896</v>
       </c>
       <c r="K49" t="n">
-        <v>1.554300285995806e-06</v>
+        <v>0.01172125493550799</v>
       </c>
     </row>
     <row r="50">
@@ -4112,34 +4112,34 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ice</t>
+          <t>heating_rate_C_min</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>Heating rate</t>
         </is>
       </c>
       <c r="E50" t="n">
-        <v>565</v>
+        <v>365</v>
       </c>
       <c r="F50" t="n">
-        <v>0.04355857131875047</v>
+        <v>0.01629854084767973</v>
       </c>
       <c r="G50" t="n">
-        <v>0.3013358093644102</v>
+        <v>0.7563056581858302</v>
       </c>
       <c r="H50" t="n">
-        <v>0.004728200849065525</v>
+        <v>0.0123581641819504</v>
       </c>
       <c r="I50" t="n">
-        <v>0.9107125777386065</v>
+        <v>0.8139747042176796</v>
       </c>
       <c r="J50" t="n">
-        <v>0.00386844341813936</v>
+        <v>0.01152656901910095</v>
       </c>
       <c r="K50" t="n">
-        <v>0.9105946212123319</v>
+        <v>0.8136043619314126</v>
       </c>
     </row>
     <row r="51">
@@ -4155,249 +4155,249 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>plateau_capacity_mAh_g</t>
+          <t>pore_volume_cm3_g</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Plateau capacity</t>
+          <t>Pore volume</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>565</v>
+        <v>302</v>
       </c>
       <c r="F51" t="n">
-        <v>-0.06836103203017327</v>
+        <v>-0.07074629617880276</v>
       </c>
       <c r="G51" t="n">
-        <v>0.1045415610114413</v>
+        <v>0.2202447204383185</v>
       </c>
       <c r="H51" t="n">
-        <v>-0.0730458988426357</v>
+        <v>-0.09180477632184833</v>
       </c>
       <c r="I51" t="n">
-        <v>0.08278439846914021</v>
+        <v>0.1113521838275141</v>
       </c>
       <c r="J51" t="n">
-        <v>-0.06066243055207192</v>
+        <v>-0.075230627298839</v>
       </c>
       <c r="K51" t="n">
-        <v>0.08278616230816543</v>
+        <v>0.1112155362240629</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>current_density_mA_g</t>
+          <t>electrolyte_type</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Current density</t>
+          <t>Electrolyte type</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>carbonization_time_h</t>
+          <t>lc_nm</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Carbonization time</t>
+          <t>Lc</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>524</v>
+        <v>286</v>
       </c>
       <c r="F52" t="n">
-        <v>0.03831463295276165</v>
+        <v>-0.09781715798135984</v>
       </c>
       <c r="G52" t="n">
-        <v>0.3814167157524654</v>
+        <v>0.09874776382654843</v>
       </c>
       <c r="H52" t="n">
-        <v>-0.02933874261750504</v>
+        <v>-0.1641349420705074</v>
       </c>
       <c r="I52" t="n">
-        <v>0.5027717774703098</v>
+        <v>0.005393974357511183</v>
       </c>
       <c r="J52" t="n">
-        <v>-0.02493620839246706</v>
+        <v>-0.1345304650379796</v>
       </c>
       <c r="K52" t="n">
-        <v>0.4903975758835577</v>
+        <v>0.005589871837256947</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>current_density_mA_g</t>
+          <t>electrolyte_type</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Current density</t>
+          <t>Electrolyte type</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>heating_rate_C_min</t>
+          <t>la_nm</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Heating rate</t>
+          <t>La</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>365</v>
+        <v>256</v>
       </c>
       <c r="F53" t="n">
-        <v>0.02787006739051085</v>
+        <v>-0.2283888372891541</v>
       </c>
       <c r="G53" t="n">
-        <v>0.5956033750771572</v>
+        <v>0.0002285568410490067</v>
       </c>
       <c r="H53" t="n">
-        <v>0.1803871150965151</v>
+        <v>-0.3008459514899685</v>
       </c>
       <c r="I53" t="n">
-        <v>0.0005343491194051549</v>
+        <v>9.387539543675841e-07</v>
       </c>
       <c r="J53" t="n">
-        <v>0.143569388929301</v>
+        <v>-0.2462639562527961</v>
       </c>
       <c r="K53" t="n">
-        <v>0.0009858805195212237</v>
+        <v>1.554300285995806e-06</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>current_density_mA_g</t>
+          <t>electrolyte_type</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Current density</t>
+          <t>Electrolyte type</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>pore_volume_cm3_g</t>
+          <t>ice</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Pore volume</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="E54" t="n">
-        <v>302</v>
+        <v>565</v>
       </c>
       <c r="F54" t="n">
-        <v>0.3576647506410962</v>
+        <v>0.04355857131875049</v>
       </c>
       <c r="G54" t="n">
-        <v>1.525384041610665e-10</v>
+        <v>0.3013358093644102</v>
       </c>
       <c r="H54" t="n">
-        <v>0.324968632919931</v>
+        <v>0.004728200849065525</v>
       </c>
       <c r="I54" t="n">
-        <v>7.399106522941429e-09</v>
+        <v>0.9107125777386066</v>
       </c>
       <c r="J54" t="n">
-        <v>0.2369064785528564</v>
+        <v>0.00386844341813936</v>
       </c>
       <c r="K54" t="n">
-        <v>1.640981083241035e-08</v>
+        <v>0.9105946212123319</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>current_density_mA_g</t>
+          <t>electrolyte_type</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Current density</t>
+          <t>Electrolyte type</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>lc_nm</t>
+          <t>plateau_capacity_mAh_g</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Lc</t>
+          <t>Plateau capacity</t>
         </is>
       </c>
       <c r="E55" t="n">
-        <v>286</v>
+        <v>565</v>
       </c>
       <c r="F55" t="n">
-        <v>-0.1296943028191048</v>
+        <v>-0.06836103203017323</v>
       </c>
       <c r="G55" t="n">
-        <v>0.02830778545923418</v>
+        <v>0.1045415610114413</v>
       </c>
       <c r="H55" t="n">
-        <v>-0.0896920567533592</v>
+        <v>-0.0730458988426357</v>
       </c>
       <c r="I55" t="n">
-        <v>0.1302189921701688</v>
+        <v>0.08278439846914018</v>
       </c>
       <c r="J55" t="n">
-        <v>-0.06138490027637567</v>
+        <v>-0.06066243055207192</v>
       </c>
       <c r="K55" t="n">
-        <v>0.1524666013719151</v>
+        <v>0.08278616230816543</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>current_density_mA_g</t>
+          <t>electrolyte_type</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Current density</t>
+          <t>Electrolyte type</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>la_nm</t>
+          <t>reversible_capacity_mAh_g</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>La</t>
+          <t>Reversible capacity</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>256</v>
+        <v>558</v>
       </c>
       <c r="F56" t="n">
-        <v>-0.2510935046479174</v>
+        <v>-0.1188996873334528</v>
       </c>
       <c r="G56" t="n">
-        <v>4.84214203994799e-05</v>
+        <v>0.004918319928076042</v>
       </c>
       <c r="H56" t="n">
-        <v>-0.178569296820862</v>
+        <v>-0.1245552216711147</v>
       </c>
       <c r="I56" t="n">
-        <v>0.004154330651809216</v>
+        <v>0.003207353606992277</v>
       </c>
       <c r="J56" t="n">
-        <v>-0.1162547786461695</v>
+        <v>-0.1018432975273344</v>
       </c>
       <c r="K56" t="n">
-        <v>0.01046828569769067</v>
+        <v>0.003286268872573505</v>
       </c>
     </row>
     <row r="57">
@@ -4413,34 +4413,34 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ice</t>
+          <t>carbonization_time_h</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>Carbonization time</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>565</v>
+        <v>524</v>
       </c>
       <c r="F57" t="n">
-        <v>-0.3690072488853919</v>
+        <v>0.03831463295276165</v>
       </c>
       <c r="G57" t="n">
-        <v>1.147596633470949e-19</v>
+        <v>0.3814167157524654</v>
       </c>
       <c r="H57" t="n">
-        <v>-0.415048803888323</v>
+        <v>-0.02933874261750504</v>
       </c>
       <c r="I57" t="n">
-        <v>6.181682170482473e-25</v>
+        <v>0.5027717774703095</v>
       </c>
       <c r="J57" t="n">
-        <v>-0.3020176467713795</v>
+        <v>-0.02493620839246706</v>
       </c>
       <c r="K57" t="n">
-        <v>5.49800343820078e-23</v>
+        <v>0.4903975758835577</v>
       </c>
     </row>
     <row r="58">
@@ -4456,690 +4456,690 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>plateau_capacity_mAh_g</t>
+          <t>heating_rate_C_min</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Plateau capacity</t>
+          <t>Heating rate</t>
         </is>
       </c>
       <c r="E58" t="n">
-        <v>565</v>
+        <v>365</v>
       </c>
       <c r="F58" t="n">
-        <v>-0.3027342881133855</v>
+        <v>0.0278700673905108</v>
       </c>
       <c r="G58" t="n">
-        <v>1.934925644684882e-13</v>
+        <v>0.5956033750771572</v>
       </c>
       <c r="H58" t="n">
-        <v>-0.383720220884475</v>
+        <v>0.1803871150965151</v>
       </c>
       <c r="I58" t="n">
-        <v>2.922212254704598e-21</v>
+        <v>0.0005343491194051567</v>
       </c>
       <c r="J58" t="n">
-        <v>-0.2843105059157303</v>
+        <v>0.143569388929301</v>
       </c>
       <c r="K58" t="n">
-        <v>5.39462263205365e-20</v>
+        <v>0.0009858805195212237</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>carbonization_time_h</t>
+          <t>current_density_mA_g</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Carbonization time</t>
+          <t>Current density</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>heating_rate_C_min</t>
+          <t>pore_volume_cm3_g</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Heating rate</t>
+          <t>Pore volume</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>348</v>
+        <v>302</v>
       </c>
       <c r="F59" t="n">
-        <v>-0.1106388191475568</v>
+        <v>0.3576647506410963</v>
       </c>
       <c r="G59" t="n">
-        <v>0.03912673234466769</v>
+        <v>1.525384041610665e-10</v>
       </c>
       <c r="H59" t="n">
-        <v>-0.2364199653184904</v>
+        <v>0.324968632919931</v>
       </c>
       <c r="I59" t="n">
-        <v>8.278824341034292e-06</v>
+        <v>7.399106522941446e-09</v>
       </c>
       <c r="J59" t="n">
-        <v>-0.2085178985473644</v>
+        <v>0.2369064785528564</v>
       </c>
       <c r="K59" t="n">
-        <v>7.1144612260661e-06</v>
+        <v>1.640981083241035e-08</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>carbonization_time_h</t>
+          <t>current_density_mA_g</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Carbonization time</t>
+          <t>Current density</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>pore_volume_cm3_g</t>
+          <t>lc_nm</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Pore volume</t>
+          <t>Lc</t>
         </is>
       </c>
       <c r="E60" t="n">
-        <v>278</v>
+        <v>286</v>
       </c>
       <c r="F60" t="n">
-        <v>-0.05046364497890993</v>
+        <v>-0.1296943028191048</v>
       </c>
       <c r="G60" t="n">
-        <v>0.4019519968796342</v>
+        <v>0.0283077854592339</v>
       </c>
       <c r="H60" t="n">
-        <v>-0.02362842107151205</v>
+        <v>-0.0896920567533592</v>
       </c>
       <c r="I60" t="n">
-        <v>0.694877802167282</v>
+        <v>0.1302189921701688</v>
       </c>
       <c r="J60" t="n">
-        <v>-0.01855372898498633</v>
+        <v>-0.06138490027637567</v>
       </c>
       <c r="K60" t="n">
-        <v>0.6890878231267816</v>
+        <v>0.1524666013719151</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>carbonization_time_h</t>
+          <t>current_density_mA_g</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Carbonization time</t>
+          <t>Current density</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>lc_nm</t>
+          <t>la_nm</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Lc</t>
+          <t>La</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="F61" t="n">
-        <v>-0.1577998662138713</v>
+        <v>-0.2510935046479174</v>
       </c>
       <c r="G61" t="n">
-        <v>0.01067644863229665</v>
+        <v>4.84214203994799e-05</v>
       </c>
       <c r="H61" t="n">
-        <v>0.007087163510345731</v>
+        <v>-0.178569296820862</v>
       </c>
       <c r="I61" t="n">
-        <v>0.9092786236185226</v>
+        <v>0.004154330651809222</v>
       </c>
       <c r="J61" t="n">
-        <v>0.01272511439833879</v>
+        <v>-0.1162547786461695</v>
       </c>
       <c r="K61" t="n">
-        <v>0.789247927917908</v>
+        <v>0.01046828569769067</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>carbonization_time_h</t>
+          <t>current_density_mA_g</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Carbonization time</t>
+          <t>Current density</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>la_nm</t>
+          <t>ice</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>La</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="E62" t="n">
-        <v>230</v>
+        <v>565</v>
       </c>
       <c r="F62" t="n">
-        <v>-0.2858571099025972</v>
+        <v>-0.3690072488853919</v>
       </c>
       <c r="G62" t="n">
-        <v>1.063420509561472e-05</v>
+        <v>1.147596633470949e-19</v>
       </c>
       <c r="H62" t="n">
-        <v>-0.412272619466077</v>
+        <v>-0.415048803888323</v>
       </c>
       <c r="I62" t="n">
-        <v>7.504132286295331e-11</v>
+        <v>6.181682170482455e-25</v>
       </c>
       <c r="J62" t="n">
-        <v>-0.3223103086676418</v>
+        <v>-0.3020176467713795</v>
       </c>
       <c r="K62" t="n">
-        <v>1.965515925541108e-10</v>
+        <v>5.49800343820078e-23</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>carbonization_time_h</t>
+          <t>current_density_mA_g</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Carbonization time</t>
+          <t>Current density</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>ice</t>
+          <t>plateau_capacity_mAh_g</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>Plateau capacity</t>
         </is>
       </c>
       <c r="E63" t="n">
-        <v>524</v>
+        <v>565</v>
       </c>
       <c r="F63" t="n">
-        <v>-0.06742782742250555</v>
+        <v>-0.3027342881133855</v>
       </c>
       <c r="G63" t="n">
-        <v>0.1231800014169101</v>
+        <v>1.934925644684882e-13</v>
       </c>
       <c r="H63" t="n">
-        <v>-0.1371074757307379</v>
+        <v>-0.383720220884475</v>
       </c>
       <c r="I63" t="n">
-        <v>0.001655725342267778</v>
+        <v>2.922212254704603e-21</v>
       </c>
       <c r="J63" t="n">
-        <v>-0.1045695793933987</v>
+        <v>-0.2843105059157303</v>
       </c>
       <c r="K63" t="n">
-        <v>0.001682642436966277</v>
+        <v>5.39462263205365e-20</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>carbonization_time_h</t>
+          <t>current_density_mA_g</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Carbonization time</t>
+          <t>Current density</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>plateau_capacity_mAh_g</t>
+          <t>reversible_capacity_mAh_g</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Plateau capacity</t>
+          <t>Reversible capacity</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>524</v>
+        <v>558</v>
       </c>
       <c r="F64" t="n">
-        <v>-0.1040400056091798</v>
+        <v>-0.09047145406026903</v>
       </c>
       <c r="G64" t="n">
-        <v>0.01720181667019006</v>
+        <v>0.03262159765593155</v>
       </c>
       <c r="H64" t="n">
-        <v>-0.1524472207635033</v>
+        <v>-0.06453100911789136</v>
       </c>
       <c r="I64" t="n">
-        <v>0.0004620720505100557</v>
+        <v>0.1278783533947267</v>
       </c>
       <c r="J64" t="n">
-        <v>-0.1151604344752149</v>
+        <v>-0.04342468456778356</v>
       </c>
       <c r="K64" t="n">
-        <v>0.0006455175499470531</v>
+        <v>0.1582625986334978</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
+          <t>carbonization_time_h</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Carbonization time</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
           <t>heating_rate_C_min</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
+      <c r="D65" t="inlineStr">
         <is>
           <t>Heating rate</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>pore_volume_cm3_g</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>Pore volume</t>
-        </is>
-      </c>
       <c r="E65" t="n">
-        <v>206</v>
+        <v>348</v>
       </c>
       <c r="F65" t="n">
-        <v>0.03654999686644903</v>
+        <v>-0.1106388191475569</v>
       </c>
       <c r="G65" t="n">
-        <v>0.6019674247830828</v>
+        <v>0.03912673234466769</v>
       </c>
       <c r="H65" t="n">
-        <v>-0.02640188506999511</v>
+        <v>-0.2364199653184904</v>
       </c>
       <c r="I65" t="n">
-        <v>0.7063979079709202</v>
+        <v>8.278824341034311e-06</v>
       </c>
       <c r="J65" t="n">
-        <v>-0.02098190133162098</v>
+        <v>-0.2085178985473644</v>
       </c>
       <c r="K65" t="n">
-        <v>0.6935357457408117</v>
+        <v>7.1144612260661e-06</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>heating_rate_C_min</t>
+          <t>carbonization_time_h</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Heating rate</t>
+          <t>Carbonization time</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>lc_nm</t>
+          <t>pore_volume_cm3_g</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Lc</t>
+          <t>Pore volume</t>
         </is>
       </c>
       <c r="E66" t="n">
-        <v>168</v>
+        <v>278</v>
       </c>
       <c r="F66" t="n">
-        <v>-0.01489999487612455</v>
+        <v>-0.05046364497890994</v>
       </c>
       <c r="G66" t="n">
-        <v>0.8479813155139151</v>
+        <v>0.4019519968796342</v>
       </c>
       <c r="H66" t="n">
-        <v>-0.1403970268274069</v>
+        <v>-0.02362842107151205</v>
       </c>
       <c r="I66" t="n">
-        <v>0.06949804417675659</v>
+        <v>0.6948778021672821</v>
       </c>
       <c r="J66" t="n">
-        <v>-0.103566199773595</v>
+        <v>-0.01855372898498633</v>
       </c>
       <c r="K66" t="n">
-        <v>0.08174071250632295</v>
+        <v>0.6890878231267816</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>heating_rate_C_min</t>
+          <t>carbonization_time_h</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Heating rate</t>
+          <t>Carbonization time</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>la_nm</t>
+          <t>lc_nm</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>La</t>
+          <t>Lc</t>
         </is>
       </c>
       <c r="E67" t="n">
-        <v>146</v>
+        <v>261</v>
       </c>
       <c r="F67" t="n">
-        <v>-0.01206984641721954</v>
+        <v>-0.1577998662138713</v>
       </c>
       <c r="G67" t="n">
-        <v>0.8850328627914015</v>
+        <v>0.01067644863229665</v>
       </c>
       <c r="H67" t="n">
-        <v>0.02366403198360413</v>
+        <v>0.007087163510345731</v>
       </c>
       <c r="I67" t="n">
-        <v>0.7767816743698485</v>
+        <v>0.9092786236185226</v>
       </c>
       <c r="J67" t="n">
-        <v>0.02504588065536022</v>
+        <v>0.01272511439833879</v>
       </c>
       <c r="K67" t="n">
-        <v>0.6936126835711451</v>
+        <v>0.789247927917908</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>heating_rate_C_min</t>
+          <t>carbonization_time_h</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Heating rate</t>
+          <t>Carbonization time</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>ice</t>
+          <t>la_nm</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>La</t>
         </is>
       </c>
       <c r="E68" t="n">
-        <v>365</v>
+        <v>230</v>
       </c>
       <c r="F68" t="n">
-        <v>-0.1029170753002386</v>
+        <v>-0.2858571099025972</v>
       </c>
       <c r="G68" t="n">
-        <v>0.04944856133872348</v>
+        <v>1.063420509561472e-05</v>
       </c>
       <c r="H68" t="n">
-        <v>-0.05809852362754963</v>
+        <v>-0.412272619466077</v>
       </c>
       <c r="I68" t="n">
-        <v>0.268251200131539</v>
+        <v>7.504132286295316e-11</v>
       </c>
       <c r="J68" t="n">
-        <v>-0.0441530581841631</v>
+        <v>-0.3223103086676418</v>
       </c>
       <c r="K68" t="n">
-        <v>0.2698342777507923</v>
+        <v>1.965515925541108e-10</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>heating_rate_C_min</t>
+          <t>carbonization_time_h</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Heating rate</t>
+          <t>Carbonization time</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>plateau_capacity_mAh_g</t>
+          <t>ice</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Plateau capacity</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="E69" t="n">
-        <v>365</v>
+        <v>524</v>
       </c>
       <c r="F69" t="n">
-        <v>-0.1063011190770503</v>
+        <v>-0.06742782742250554</v>
       </c>
       <c r="G69" t="n">
-        <v>0.04239028934904038</v>
+        <v>0.1231800014169101</v>
       </c>
       <c r="H69" t="n">
-        <v>-0.0816822071140134</v>
+        <v>-0.1371074757307379</v>
       </c>
       <c r="I69" t="n">
-        <v>0.1192835859700816</v>
+        <v>0.001655725342267775</v>
       </c>
       <c r="J69" t="n">
-        <v>-0.06363017915856511</v>
+        <v>-0.1045695793933987</v>
       </c>
       <c r="K69" t="n">
-        <v>0.1185844558379846</v>
+        <v>0.001682642436966277</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>pore_volume_cm3_g</t>
+          <t>carbonization_time_h</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Pore volume</t>
+          <t>Carbonization time</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>lc_nm</t>
+          <t>plateau_capacity_mAh_g</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Lc</t>
+          <t>Plateau capacity</t>
         </is>
       </c>
       <c r="E70" t="n">
-        <v>154</v>
+        <v>524</v>
       </c>
       <c r="F70" t="n">
-        <v>-0.1588720716853017</v>
+        <v>-0.1040400056091798</v>
       </c>
       <c r="G70" t="n">
-        <v>0.0490674173520891</v>
+        <v>0.01720181667019006</v>
       </c>
       <c r="H70" t="n">
-        <v>-0.2236777355799165</v>
+        <v>-0.1524472207635033</v>
       </c>
       <c r="I70" t="n">
-        <v>0.005294061189543539</v>
+        <v>0.0004620720505100558</v>
       </c>
       <c r="J70" t="n">
-        <v>-0.1558397838259867</v>
+        <v>-0.1151604344752149</v>
       </c>
       <c r="K70" t="n">
-        <v>0.004285701784196834</v>
+        <v>0.0006455175499470531</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>pore_volume_cm3_g</t>
+          <t>carbonization_time_h</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Pore volume</t>
+          <t>Carbonization time</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>la_nm</t>
+          <t>reversible_capacity_mAh_g</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>La</t>
+          <t>Reversible capacity</t>
         </is>
       </c>
       <c r="E71" t="n">
-        <v>134</v>
+        <v>522</v>
       </c>
       <c r="F71" t="n">
-        <v>-0.1643863545268226</v>
+        <v>-0.0672773009919016</v>
       </c>
       <c r="G71" t="n">
-        <v>0.05769410188076184</v>
+        <v>0.1247443323507617</v>
       </c>
       <c r="H71" t="n">
-        <v>-0.232388658227857</v>
+        <v>-0.08394786251005039</v>
       </c>
       <c r="I71" t="n">
-        <v>0.006892673648307064</v>
+        <v>0.05526713546806346</v>
       </c>
       <c r="J71" t="n">
-        <v>-0.160941694456608</v>
+        <v>-0.06238665039041275</v>
       </c>
       <c r="K71" t="n">
-        <v>0.005977676324213304</v>
+        <v>0.06124436948341461</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
+          <t>heating_rate_C_min</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Heating rate</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
           <t>pore_volume_cm3_g</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr">
+      <c r="D72" t="inlineStr">
         <is>
           <t>Pore volume</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>ice</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>ICE</t>
-        </is>
-      </c>
       <c r="E72" t="n">
-        <v>302</v>
+        <v>206</v>
       </c>
       <c r="F72" t="n">
-        <v>-0.6303280702605111</v>
+        <v>0.03654999686644902</v>
       </c>
       <c r="G72" t="n">
-        <v>7.499254830415694e-35</v>
+        <v>0.6019674247830828</v>
       </c>
       <c r="H72" t="n">
-        <v>-0.6933427652186777</v>
+        <v>-0.02640188506999511</v>
       </c>
       <c r="I72" t="n">
-        <v>1.349719311522128e-44</v>
+        <v>0.7063979079709201</v>
       </c>
       <c r="J72" t="n">
-        <v>-0.514946747902482</v>
+        <v>-0.02098190133162098</v>
       </c>
       <c r="K72" t="n">
-        <v>2.000925863129017e-40</v>
+        <v>0.6935357457408117</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>pore_volume_cm3_g</t>
+          <t>heating_rate_C_min</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Pore volume</t>
+          <t>Heating rate</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>plateau_capacity_mAh_g</t>
+          <t>lc_nm</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Plateau capacity</t>
+          <t>Lc</t>
         </is>
       </c>
       <c r="E73" t="n">
-        <v>302</v>
+        <v>168</v>
       </c>
       <c r="F73" t="n">
-        <v>-0.5068825166502335</v>
+        <v>-0.01489999487612455</v>
       </c>
       <c r="G73" t="n">
-        <v>4.059895449149044e-21</v>
+        <v>0.8479813155139151</v>
       </c>
       <c r="H73" t="n">
-        <v>-0.6543601829456029</v>
+        <v>-0.1403970268274069</v>
       </c>
       <c r="I73" t="n">
-        <v>2.712540233230457e-38</v>
+        <v>0.06949804417675656</v>
       </c>
       <c r="J73" t="n">
-        <v>-0.4830633699933283</v>
+        <v>-0.103566199773595</v>
       </c>
       <c r="K73" t="n">
-        <v>1.858722389360642e-34</v>
+        <v>0.08174071250632295</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>lc_nm</t>
+          <t>heating_rate_C_min</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Lc</t>
+          <t>Heating rate</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -5153,36 +5153,36 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>243</v>
+        <v>146</v>
       </c>
       <c r="F74" t="n">
-        <v>0.484737221869695</v>
+        <v>-0.01206984641721954</v>
       </c>
       <c r="G74" t="n">
-        <v>1.00595944823409e-15</v>
+        <v>0.8850328627914015</v>
       </c>
       <c r="H74" t="n">
-        <v>0.2793962737626825</v>
+        <v>0.02366403198360413</v>
       </c>
       <c r="I74" t="n">
-        <v>9.812489414764302e-06</v>
+        <v>0.7767816743698485</v>
       </c>
       <c r="J74" t="n">
-        <v>0.2004743231536769</v>
+        <v>0.02504588065536022</v>
       </c>
       <c r="K74" t="n">
-        <v>3.461284516749348e-06</v>
+        <v>0.6936126835711451</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>lc_nm</t>
+          <t>heating_rate_C_min</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Lc</t>
+          <t>Heating rate</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -5196,36 +5196,36 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>286</v>
+        <v>365</v>
       </c>
       <c r="F75" t="n">
-        <v>0.1883759717344395</v>
+        <v>-0.1029170753002386</v>
       </c>
       <c r="G75" t="n">
-        <v>0.001372009608555396</v>
+        <v>0.04944856133872348</v>
       </c>
       <c r="H75" t="n">
-        <v>0.1025869439101235</v>
+        <v>-0.05809852362754963</v>
       </c>
       <c r="I75" t="n">
-        <v>0.08329551112644691</v>
+        <v>0.2682512001315391</v>
       </c>
       <c r="J75" t="n">
-        <v>0.0710620341866106</v>
+        <v>-0.0441530581841631</v>
       </c>
       <c r="K75" t="n">
-        <v>0.07407415486138647</v>
+        <v>0.2698342777507923</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>lc_nm</t>
+          <t>heating_rate_C_min</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Lc</t>
+          <t>Heating rate</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -5239,154 +5239,713 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>286</v>
+        <v>365</v>
       </c>
       <c r="F76" t="n">
-        <v>0.15000067156804</v>
+        <v>-0.1063011190770503</v>
       </c>
       <c r="G76" t="n">
-        <v>0.01108464860441246</v>
+        <v>0.04239028934904038</v>
       </c>
       <c r="H76" t="n">
-        <v>0.1161156691107151</v>
+        <v>-0.0816822071140134</v>
       </c>
       <c r="I76" t="n">
-        <v>0.04979336375797689</v>
+        <v>0.1192835859700817</v>
       </c>
       <c r="J76" t="n">
-        <v>0.07607623075020999</v>
+        <v>-0.06363017915856511</v>
       </c>
       <c r="K76" t="n">
-        <v>0.05680372081869858</v>
+        <v>0.1185844558379846</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>la_nm</t>
+          <t>heating_rate_C_min</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>La</t>
+          <t>Heating rate</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>ice</t>
+          <t>reversible_capacity_mAh_g</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>Reversible capacity</t>
         </is>
       </c>
       <c r="E77" t="n">
-        <v>256</v>
+        <v>363</v>
       </c>
       <c r="F77" t="n">
-        <v>0.1503119518056599</v>
+        <v>-0.01711886018273929</v>
       </c>
       <c r="G77" t="n">
-        <v>0.01608804321031551</v>
+        <v>0.7451379352274501</v>
       </c>
       <c r="H77" t="n">
-        <v>0.1681245669226088</v>
+        <v>-0.07803991550431574</v>
       </c>
       <c r="I77" t="n">
-        <v>0.007016796862992602</v>
+        <v>0.1378100006859607</v>
       </c>
       <c r="J77" t="n">
-        <v>0.1171416007417869</v>
+        <v>-0.05943436567619537</v>
       </c>
       <c r="K77" t="n">
-        <v>0.005309156051810144</v>
+        <v>0.138429594579151</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>la_nm</t>
+          <t>pore_volume_cm3_g</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>La</t>
+          <t>Pore volume</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>plateau_capacity_mAh_g</t>
+          <t>lc_nm</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Plateau capacity</t>
+          <t>Lc</t>
         </is>
       </c>
       <c r="E78" t="n">
-        <v>256</v>
+        <v>154</v>
       </c>
       <c r="F78" t="n">
-        <v>0.2266734618594218</v>
+        <v>-0.1588720716853017</v>
       </c>
       <c r="G78" t="n">
-        <v>0.0002554454456974599</v>
+        <v>0.0490674173520891</v>
       </c>
       <c r="H78" t="n">
-        <v>0.231154352351584</v>
+        <v>-0.2236777355799165</v>
       </c>
       <c r="I78" t="n">
-        <v>0.0001907017655417267</v>
+        <v>0.005294061189543539</v>
       </c>
       <c r="J78" t="n">
-        <v>0.1625391139401165</v>
+        <v>-0.1558397838259867</v>
       </c>
       <c r="K78" t="n">
-        <v>0.0001127405095644972</v>
+        <v>0.004285701784196834</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
+          <t>pore_volume_cm3_g</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Pore volume</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>la_nm</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>La</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>134</v>
+      </c>
+      <c r="F79" t="n">
+        <v>-0.1643863545268227</v>
+      </c>
+      <c r="G79" t="n">
+        <v>0.05769410188076184</v>
+      </c>
+      <c r="H79" t="n">
+        <v>-0.232388658227857</v>
+      </c>
+      <c r="I79" t="n">
+        <v>0.00689267364830707</v>
+      </c>
+      <c r="J79" t="n">
+        <v>-0.160941694456608</v>
+      </c>
+      <c r="K79" t="n">
+        <v>0.005977676324213304</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>pore_volume_cm3_g</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Pore volume</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
           <t>ice</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr">
+      <c r="D80" t="inlineStr">
         <is>
           <t>ICE</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr">
+      <c r="E80" t="n">
+        <v>302</v>
+      </c>
+      <c r="F80" t="n">
+        <v>-0.6303280702605111</v>
+      </c>
+      <c r="G80" t="n">
+        <v>7.499254830415694e-35</v>
+      </c>
+      <c r="H80" t="n">
+        <v>-0.6933427652186777</v>
+      </c>
+      <c r="I80" t="n">
+        <v>1.349719311522112e-44</v>
+      </c>
+      <c r="J80" t="n">
+        <v>-0.514946747902482</v>
+      </c>
+      <c r="K80" t="n">
+        <v>2.000925863129017e-40</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>pore_volume_cm3_g</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Pore volume</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
         <is>
           <t>plateau_capacity_mAh_g</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr">
+      <c r="D81" t="inlineStr">
         <is>
           <t>Plateau capacity</t>
         </is>
       </c>
-      <c r="E79" t="n">
+      <c r="E81" t="n">
+        <v>302</v>
+      </c>
+      <c r="F81" t="n">
+        <v>-0.5068825166502333</v>
+      </c>
+      <c r="G81" t="n">
+        <v>4.059895449149229e-21</v>
+      </c>
+      <c r="H81" t="n">
+        <v>-0.6543601829456029</v>
+      </c>
+      <c r="I81" t="n">
+        <v>2.712540233230541e-38</v>
+      </c>
+      <c r="J81" t="n">
+        <v>-0.4830633699933283</v>
+      </c>
+      <c r="K81" t="n">
+        <v>1.858722389360642e-34</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>pore_volume_cm3_g</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Pore volume</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>reversible_capacity_mAh_g</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Reversible capacity</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>302</v>
+      </c>
+      <c r="F82" t="n">
+        <v>-0.01706843989641395</v>
+      </c>
+      <c r="G82" t="n">
+        <v>0.7676812177314141</v>
+      </c>
+      <c r="H82" t="n">
+        <v>-0.1409711928463241</v>
+      </c>
+      <c r="I82" t="n">
+        <v>0.01420981371112535</v>
+      </c>
+      <c r="J82" t="n">
+        <v>-0.1031195340081671</v>
+      </c>
+      <c r="K82" t="n">
+        <v>0.007664687330225455</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>lc_nm</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Lc</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>la_nm</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>La</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>243</v>
+      </c>
+      <c r="F83" t="n">
+        <v>0.4847372218696949</v>
+      </c>
+      <c r="G83" t="n">
+        <v>1.00595944823409e-15</v>
+      </c>
+      <c r="H83" t="n">
+        <v>0.2793962737626825</v>
+      </c>
+      <c r="I83" t="n">
+        <v>9.812489414764271e-06</v>
+      </c>
+      <c r="J83" t="n">
+        <v>0.2004743231536769</v>
+      </c>
+      <c r="K83" t="n">
+        <v>3.461284516749348e-06</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>lc_nm</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Lc</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>ice</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>ICE</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>286</v>
+      </c>
+      <c r="F84" t="n">
+        <v>0.1883759717344396</v>
+      </c>
+      <c r="G84" t="n">
+        <v>0.001372009608555396</v>
+      </c>
+      <c r="H84" t="n">
+        <v>0.1025869439101235</v>
+      </c>
+      <c r="I84" t="n">
+        <v>0.0832955111264469</v>
+      </c>
+      <c r="J84" t="n">
+        <v>0.0710620341866106</v>
+      </c>
+      <c r="K84" t="n">
+        <v>0.07407415486138647</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>lc_nm</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Lc</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>plateau_capacity_mAh_g</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Plateau capacity</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>286</v>
+      </c>
+      <c r="F85" t="n">
+        <v>0.15000067156804</v>
+      </c>
+      <c r="G85" t="n">
+        <v>0.01108464860441246</v>
+      </c>
+      <c r="H85" t="n">
+        <v>0.1161156691107151</v>
+      </c>
+      <c r="I85" t="n">
+        <v>0.04979336375797688</v>
+      </c>
+      <c r="J85" t="n">
+        <v>0.07607623075020999</v>
+      </c>
+      <c r="K85" t="n">
+        <v>0.05680372081869858</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>lc_nm</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Lc</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>reversible_capacity_mAh_g</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Reversible capacity</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>286</v>
+      </c>
+      <c r="F86" t="n">
+        <v>-0.05898962704023292</v>
+      </c>
+      <c r="G86" t="n">
+        <v>0.3201731624811084</v>
+      </c>
+      <c r="H86" t="n">
+        <v>0.005101546805135119</v>
+      </c>
+      <c r="I86" t="n">
+        <v>0.9315477342078475</v>
+      </c>
+      <c r="J86" t="n">
+        <v>0.002853877850494505</v>
+      </c>
+      <c r="K86" t="n">
+        <v>0.942787132614611</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>la_nm</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>La</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>ice</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>ICE</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>256</v>
+      </c>
+      <c r="F87" t="n">
+        <v>0.15031195180566</v>
+      </c>
+      <c r="G87" t="n">
+        <v>0.01608804321031551</v>
+      </c>
+      <c r="H87" t="n">
+        <v>0.1681245669226088</v>
+      </c>
+      <c r="I87" t="n">
+        <v>0.007016796862992614</v>
+      </c>
+      <c r="J87" t="n">
+        <v>0.1171416007417869</v>
+      </c>
+      <c r="K87" t="n">
+        <v>0.005309156051810144</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>la_nm</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>La</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>plateau_capacity_mAh_g</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Plateau capacity</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>256</v>
+      </c>
+      <c r="F88" t="n">
+        <v>0.2266734618594217</v>
+      </c>
+      <c r="G88" t="n">
+        <v>0.0002554454456974599</v>
+      </c>
+      <c r="H88" t="n">
+        <v>0.231154352351584</v>
+      </c>
+      <c r="I88" t="n">
+        <v>0.0001907017655417275</v>
+      </c>
+      <c r="J88" t="n">
+        <v>0.1625391139401165</v>
+      </c>
+      <c r="K88" t="n">
+        <v>0.0001127405095644972</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>la_nm</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>La</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>reversible_capacity_mAh_g</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Reversible capacity</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>256</v>
+      </c>
+      <c r="F89" t="n">
+        <v>0.09292254067767891</v>
+      </c>
+      <c r="G89" t="n">
+        <v>0.1381556029752343</v>
+      </c>
+      <c r="H89" t="n">
+        <v>0.1560186516401053</v>
+      </c>
+      <c r="I89" t="n">
+        <v>0.01244015379119675</v>
+      </c>
+      <c r="J89" t="n">
+        <v>0.1076073620138166</v>
+      </c>
+      <c r="K89" t="n">
+        <v>0.01040846123393323</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>ice</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>ICE</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>plateau_capacity_mAh_g</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Plateau capacity</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
         <v>565</v>
       </c>
-      <c r="F79" t="n">
-        <v>0.8071984501983951</v>
-      </c>
-      <c r="G79" t="n">
-        <v>5.307129168221488e-131</v>
-      </c>
-      <c r="H79" t="n">
+      <c r="F90" t="n">
+        <v>0.8071984501983953</v>
+      </c>
+      <c r="G90" t="n">
+        <v>5.307129168219949e-131</v>
+      </c>
+      <c r="H90" t="n">
         <v>0.8195196049301859</v>
       </c>
-      <c r="I79" t="n">
-        <v>2.988374690670115e-138</v>
-      </c>
-      <c r="J79" t="n">
+      <c r="I90" t="n">
+        <v>2.988374690670179e-138</v>
+      </c>
+      <c r="J90" t="n">
         <v>0.6270331237351076</v>
       </c>
-      <c r="K79" t="n">
+      <c r="K90" t="n">
         <v>2.199705618186211e-106</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>ice</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>ICE</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>reversible_capacity_mAh_g</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Reversible capacity</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>558</v>
+      </c>
+      <c r="F91" t="n">
+        <v>0.2465902417690275</v>
+      </c>
+      <c r="G91" t="n">
+        <v>3.563066234117484e-09</v>
+      </c>
+      <c r="H91" t="n">
+        <v>0.311104563696373</v>
+      </c>
+      <c r="I91" t="n">
+        <v>5.484221802015e-14</v>
+      </c>
+      <c r="J91" t="n">
+        <v>0.2213721254309031</v>
+      </c>
+      <c r="K91" t="n">
+        <v>5.896322659438465e-15</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>plateau_capacity_mAh_g</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Plateau capacity</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>reversible_capacity_mAh_g</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Reversible capacity</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>558</v>
+      </c>
+      <c r="F92" t="n">
+        <v>0.3921828327621878</v>
+      </c>
+      <c r="G92" t="n">
+        <v>5.861177627278616e-22</v>
+      </c>
+      <c r="H92" t="n">
+        <v>0.4879503640505743</v>
+      </c>
+      <c r="I92" t="n">
+        <v>1.015585166334866e-34</v>
+      </c>
+      <c r="J92" t="n">
+        <v>0.3951054903466095</v>
+      </c>
+      <c r="K92" t="n">
+        <v>5.883829956401254e-43</v>
       </c>
     </row>
   </sheetData>
@@ -5400,7 +5959,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:O15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5469,6 +6028,11 @@
           <t>plateau_capacity_mAh_g</t>
         </is>
       </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>reversible_capacity_mAh_g</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -5515,6 +6079,9 @@
       <c r="N2" t="n">
         <v>0.8173875628362022</v>
       </c>
+      <c r="O2" t="n">
+        <v>0.199520482151398</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -5561,6 +6128,9 @@
       <c r="N3" t="n">
         <v>-0.07225381674120725</v>
       </c>
+      <c r="O3" t="n">
+        <v>0.06833061392295345</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -5607,6 +6177,9 @@
       <c r="N4" t="n">
         <v>0.05287409906917158</v>
       </c>
+      <c r="O4" t="n">
+        <v>-0.08927954845356459</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -5653,6 +6226,9 @@
       <c r="N5" t="n">
         <v>-0.5295537533936092</v>
       </c>
+      <c r="O5" t="n">
+        <v>-0.03846128090225403</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -5699,6 +6275,9 @@
       <c r="N6" t="n">
         <v>-0.06836103203017325</v>
       </c>
+      <c r="O6" t="n">
+        <v>-0.1188996873334529</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -5745,6 +6324,9 @@
       <c r="N7" t="n">
         <v>-0.3027342881133854</v>
       </c>
+      <c r="O7" t="n">
+        <v>-0.09047145406026884</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -5791,6 +6373,9 @@
       <c r="N8" t="n">
         <v>-0.1040400056091799</v>
       </c>
+      <c r="O8" t="n">
+        <v>-0.06727730099190135</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -5837,6 +6422,9 @@
       <c r="N9" t="n">
         <v>-0.1063011190770503</v>
       </c>
+      <c r="O9" t="n">
+        <v>-0.01711886018273925</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -5883,6 +6471,9 @@
       <c r="N10" t="n">
         <v>-0.5068825166502336</v>
       </c>
+      <c r="O10" t="n">
+        <v>-0.01706843989641409</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
@@ -5929,6 +6520,9 @@
       <c r="N11" t="n">
         <v>0.1500006715680401</v>
       </c>
+      <c r="O11" t="n">
+        <v>-0.05898962704023304</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
@@ -5975,6 +6569,9 @@
       <c r="N12" t="n">
         <v>0.2266734618594218</v>
       </c>
+      <c r="O12" t="n">
+        <v>0.09292254067767894</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
@@ -6021,6 +6618,9 @@
       <c r="N13" t="n">
         <v>0.8071984501983958</v>
       </c>
+      <c r="O13" t="n">
+        <v>0.2465902417690274</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
@@ -6065,6 +6665,58 @@
         <v>0.8071984501983958</v>
       </c>
       <c r="N14" t="n">
+        <v>1</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0.3921828327621874</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>reversible_capacity_mAh_g</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.199520482151398</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.06833061392295345</v>
+      </c>
+      <c r="D15" t="n">
+        <v>-0.08927954845356459</v>
+      </c>
+      <c r="E15" t="n">
+        <v>-0.03846128090225403</v>
+      </c>
+      <c r="F15" t="n">
+        <v>-0.1188996873334529</v>
+      </c>
+      <c r="G15" t="n">
+        <v>-0.09047145406026884</v>
+      </c>
+      <c r="H15" t="n">
+        <v>-0.06727730099190135</v>
+      </c>
+      <c r="I15" t="n">
+        <v>-0.01711886018273925</v>
+      </c>
+      <c r="J15" t="n">
+        <v>-0.01706843989641409</v>
+      </c>
+      <c r="K15" t="n">
+        <v>-0.05898962704023304</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0.09292254067767894</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0.2465902417690274</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0.3921828327621874</v>
+      </c>
+      <c r="O15" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6079,7 +6731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:O15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6148,6 +6800,11 @@
           <t>plateau_capacity_mAh_g</t>
         </is>
       </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>reversible_capacity_mAh_g</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -6194,6 +6851,9 @@
       <c r="N2" t="n">
         <v>0.8206801592553979</v>
       </c>
+      <c r="O2" t="n">
+        <v>0.2560156529428892</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -6240,6 +6900,9 @@
       <c r="N3" t="n">
         <v>-0.0440993365854058</v>
       </c>
+      <c r="O3" t="n">
+        <v>0.0928585643073357</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -6286,6 +6949,9 @@
       <c r="N4" t="n">
         <v>0.1365397438371289</v>
       </c>
+      <c r="O4" t="n">
+        <v>-0.0474789944459358</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -6332,6 +6998,9 @@
       <c r="N5" t="n">
         <v>-0.6247816345029005</v>
       </c>
+      <c r="O5" t="n">
+        <v>-0.1975504284033616</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -6378,6 +7047,9 @@
       <c r="N6" t="n">
         <v>-0.07304589884263571</v>
       </c>
+      <c r="O6" t="n">
+        <v>-0.1245552216711147</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -6424,6 +7096,9 @@
       <c r="N7" t="n">
         <v>-0.3837202208844749</v>
       </c>
+      <c r="O7" t="n">
+        <v>-0.06453100911789138</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -6470,6 +7145,9 @@
       <c r="N8" t="n">
         <v>-0.1524472207635032</v>
       </c>
+      <c r="O8" t="n">
+        <v>-0.0839478625100504</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -6516,6 +7194,9 @@
       <c r="N9" t="n">
         <v>-0.0816822071140134</v>
       </c>
+      <c r="O9" t="n">
+        <v>-0.07803991550431576</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -6562,6 +7243,9 @@
       <c r="N10" t="n">
         <v>-0.6543601829456029</v>
       </c>
+      <c r="O10" t="n">
+        <v>-0.140971192846324</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
@@ -6608,6 +7292,9 @@
       <c r="N11" t="n">
         <v>0.1161156691107151</v>
       </c>
+      <c r="O11" t="n">
+        <v>0.005101546805135119</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
@@ -6654,6 +7341,9 @@
       <c r="N12" t="n">
         <v>0.231154352351584</v>
       </c>
+      <c r="O12" t="n">
+        <v>0.1560186516401053</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
@@ -6700,6 +7390,9 @@
       <c r="N13" t="n">
         <v>0.8195196049301862</v>
       </c>
+      <c r="O13" t="n">
+        <v>0.311104563696373</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
@@ -6744,6 +7437,58 @@
         <v>0.8195196049301862</v>
       </c>
       <c r="N14" t="n">
+        <v>1</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0.4879503640505743</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>reversible_capacity_mAh_g</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.2560156529428892</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.0928585643073357</v>
+      </c>
+      <c r="D15" t="n">
+        <v>-0.0474789944459358</v>
+      </c>
+      <c r="E15" t="n">
+        <v>-0.1975504284033616</v>
+      </c>
+      <c r="F15" t="n">
+        <v>-0.1245552216711147</v>
+      </c>
+      <c r="G15" t="n">
+        <v>-0.06453100911789138</v>
+      </c>
+      <c r="H15" t="n">
+        <v>-0.0839478625100504</v>
+      </c>
+      <c r="I15" t="n">
+        <v>-0.07803991550431576</v>
+      </c>
+      <c r="J15" t="n">
+        <v>-0.140971192846324</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0.005101546805135119</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0.1560186516401053</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0.311104563696373</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0.4879503640505743</v>
+      </c>
+      <c r="O15" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>